<commit_message>
feat: implement persona-based A/B email and LinkedIn DM templates for higher outreach copy diversity
</commit_message>
<xml_diff>
--- a/output/konusarak-ogren-hr-outbound-google-sheets.xlsx
+++ b/output/konusarak-ogren-hr-outbound-google-sheets.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HR Leads" sheetId="1" r:id="R7fdfb5e621524ca2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="2" r:id="Rae35cb85105e4d5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HR Leads" sheetId="1" r:id="R2aa12f7f10b44b85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="2" r:id="R6e8121f6ab5d499e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -263,14 +263,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K2" t="str">
-        <x:v>Merhaba Ebru, Garanti BBVA icin Yetenek ve Kültür Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda global bankacilik standartlari ve dijitallesme nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global bankacilik standartlari ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Ebru, Garanti BBVA için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>Subject: Garanti BBVA ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Garanti BBVA için 2 haftalık İngilizce gelişim pilotu
 Merhaba Ebru,
-Garanti BBVA ekibinin Banking / Finance olceginde global bankacilik standartlari ve dijitallesme odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global bankacilik standartlari ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Garanti BBVA icin mantikli pilot segmentini birlikte cikaralim.
+Garanti BBVA liderlik ekibinde Yetenek ve Kültür Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -308,14 +307,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>Merhaba Bülent, Akbank icin İnsan ve Kültür Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda dijital bankacilik ve yetenek donusumu nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'dijital bankacilik ve yetenek donusumu nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Bülent, Akbank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L3" t="str">
-        <x:v>Subject: Akbank ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Akbank organizasyonel İngilizce gelişim standardı
 Merhaba Bülent,
-Akbank ekibinin Banking / Finance olceginde dijital bankacilik ve yetenek donusumu odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: dijital bankacilik ve yetenek donusumu nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Akbank icin mantikli pilot segmentini birlikte cikaralim.
+Akbank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: dijital bankacilik ve yetenek donusumu nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -353,14 +351,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>Merhaba Ali, Türkiye İş Bankası icin Genel Müdür Yardımcısı - İnsan Kaynakları Yönetimi rolunuzu gordum. Banking / Finance tarafinda kurumsal olcekte egitim standardizasyonu nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'kurumsal olcekte egitim standardizasyonu nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Ali, Türkiye İş Bankası için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L4" t="str">
-        <x:v>Subject: Türkiye İş Bankası ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Türkiye İş Bankası için 2 haftalık İngilizce gelişim pilotu
 Merhaba Ali,
-Türkiye İş Bankası ekibinin Banking / Finance olceginde kurumsal olcekte egitim standardizasyonu odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: kurumsal olcekte egitim standardizasyonu nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Türkiye İş Bankası icin mantikli pilot segmentini birlikte cikaralim.
+Türkiye İş Bankası liderlik ekibinde Genel Müdür Yardımcısı - İnsan Kaynakları Yönetimi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -398,14 +395,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K5" t="str">
-        <x:v>Merhaba Özden, Yapı Kredi icin İnsan Kaynakları ve Organizasyon Genel Müdür Yardımcısı rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Özden, Yapı Kredi genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L5" t="str">
-        <x:v>Subject: Yapı Kredi ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Yapı Kredi organizasyonel İngilizce gelişim standardı
 Merhaba Özden,
-Yapı Kredi ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Yapı Kredi icin mantikli pilot segmentini birlikte cikaralim.
+Yapı Kredi bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -443,14 +439,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K6" t="str">
-        <x:v>Merhaba Cenk, QNB Finansbank icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda dijital bankacilik ve yetenek yonetimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'dijital bankacilik ve yetenek yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Cenk, QNB Finansbank için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L6" t="str">
-        <x:v>Subject: QNB Finansbank ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: QNB Finansbank için 2 haftalık İngilizce gelişim pilotu
 Merhaba Cenk,
-QNB Finansbank ekibinin Banking / Finance olceginde dijital bankacilik ve yetenek yonetimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: dijital bankacilik ve yetenek yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede QNB Finansbank icin mantikli pilot segmentini birlikte cikaralim.
+QNB Finansbank liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -488,14 +483,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K7" t="str">
-        <x:v>Merhaba Tuba, DenizBank icin İnsan Kaynakları Grubu Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda perakende bankacilik ve dijital donusum nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'perakende bankacilik ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Tuba, DenizBank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L7" t="str">
-        <x:v>Subject: DenizBank ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: DenizBank organizasyonel İngilizce gelişim standardı
 Merhaba Tuba,
-DenizBank ekibinin Banking / Finance olceginde perakende bankacilik ve dijital donusum odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: perakende bankacilik ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede DenizBank icin mantikli pilot segmentini birlikte cikaralim.
+DenizBank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: perakende bankacilik ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -533,14 +527,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K8" t="str">
-        <x:v>Merhaba Çiğdem, TEB icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda kurumsal bankacilik ve BNP Paribas is birligi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'kurumsal bankacilik ve BNP Paribas is birligi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Çiğdem, TEB için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L8" t="str">
-        <x:v>Subject: TEB ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: TEB için 2 haftalık İngilizce gelişim pilotu
 Merhaba Çiğdem,
-TEB ekibinin Banking / Finance olceginde kurumsal bankacilik ve BNP Paribas is birligi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: kurumsal bankacilik ve BNP Paribas is birligi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede TEB icin mantikli pilot segmentini birlikte cikaralim.
+TEB liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -578,14 +571,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K9" t="str">
-        <x:v>Merhaba Hüseyin, Ziraat Bankası icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda kamu bankaciligi ve modernizasyon nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'kamu bankaciligi ve modernizasyon nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Hüseyin, Ziraat Bankası genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L9" t="str">
-        <x:v>Subject: Ziraat Bankası ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Ziraat Bankası organizasyonel İngilizce gelişim standardı
 Merhaba Hüseyin,
-Ziraat Bankası ekibinin Banking / Finance olceginde kamu bankaciligi ve modernizasyon odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: kamu bankaciligi ve modernizasyon nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Ziraat Bankası icin mantikli pilot segmentini birlikte cikaralim.
+Ziraat Bankası bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: kamu bankaciligi ve modernizasyon nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -623,14 +615,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K10" t="str">
-        <x:v>Merhaba Caner, Halkbank icin İnsan Kaynakları ve İletişim Grup Başkanı rolunuzu gordum. Banking / Finance tarafinda KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Caner, Halkbank için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L10" t="str">
-        <x:v>Subject: Halkbank ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Halkbank için 2 haftalık İngilizce gelişim pilotu
 Merhaba Caner,
-Halkbank ekibinin Banking / Finance olceginde KOBi bankaciligi ve dijitallesme odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Halkbank icin mantikli pilot segmentini birlikte cikaralim.
+Halkbank liderlik ekibinde İnsan Kaynakları ve İletişim Grup Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -668,14 +659,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>Merhaba Neşe, Halkbank icin İnsan Kaynakları Daire Başkanı rolunuzu gordum. Banking / Finance tarafinda KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Neşe, Halkbank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L11" t="str">
-        <x:v>Subject: Halkbank ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Halkbank organizasyonel İngilizce gelişim standardı
 Merhaba Neşe,
-Halkbank ekibinin Banking / Finance olceginde KOBi bankaciligi ve dijitallesme odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Halkbank icin mantikli pilot segmentini birlikte cikaralim.
+Halkbank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -713,14 +703,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K12" t="str">
-        <x:v>Merhaba Şuayyip, VakıfBank icin İnsan Kaynakları, Kurumsal Gelişim ve Performans Yönetimi GMY rolunuzu gordum. Banking / Finance tarafinda kurumsal performans ve dijital donusum nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'kurumsal performans ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Şuayyip, VakıfBank için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L12" t="str">
-        <x:v>Subject: VakıfBank ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: VakıfBank için 2 haftalık İngilizce gelişim pilotu
 Merhaba Şuayyip,
-VakıfBank ekibinin Banking / Finance olceginde kurumsal performans ve dijital donusum odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: kurumsal performans ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede VakıfBank icin mantikli pilot segmentini birlikte cikaralim.
+VakıfBank liderlik ekibinde İnsan Kaynakları, Kurumsal Gelişim ve Performans Yönetimi GMY olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -758,14 +747,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K13" t="str">
-        <x:v>Merhaba Ömer, VakıfBank icin İnsan Kaynakları Başkanı rolunuzu gordum. Banking / Finance tarafinda kurumsal performans ve dijital donusum nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'kurumsal performans ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Ömer, VakıfBank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L13" t="str">
-        <x:v>Subject: VakıfBank ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: VakıfBank organizasyonel İngilizce gelişim standardı
 Merhaba Ömer,
-VakıfBank ekibinin Banking / Finance olceginde kurumsal performans ve dijital donusum odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: kurumsal performans ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede VakıfBank icin mantikli pilot segmentini birlikte cikaralim.
+VakıfBank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: kurumsal performans ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -803,14 +791,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K14" t="str">
-        <x:v>Merhaba Hale, ING Türkiye icin İnsan Kaynakları Genel Müdür Yardımcısı ve İcra Kurulu Üyesi rolunuzu gordum. Banking / Finance tarafinda global standartlar ve dijital bankacilik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global standartlar ve dijital bankacilik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Hale, ING Türkiye için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L14" t="str">
-        <x:v>Subject: ING Türkiye ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: ING Türkiye için 2 haftalık İngilizce gelişim pilotu
 Merhaba Hale,
-ING Türkiye ekibinin Banking / Finance olceginde global standartlar ve dijital bankacilik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global standartlar ve dijital bankacilik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede ING Türkiye icin mantikli pilot segmentini birlikte cikaralim.
+ING Türkiye liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı ve İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -848,14 +835,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K15" t="str">
-        <x:v>Merhaba Funda, HSBC Türkiye icin İnsan Kaynakları ve Kurumsal İletişim Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda uluslararasi bankacilik ve global ekipler nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'uluslararasi bankacilik ve global ekipler nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Funda, HSBC Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L15" t="str">
-        <x:v>Subject: HSBC Türkiye ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: HSBC Türkiye organizasyonel İngilizce gelişim standardı
 Merhaba Funda,
-HSBC Türkiye ekibinin Banking / Finance olceginde uluslararasi bankacilik ve global ekipler odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: uluslararasi bankacilik ve global ekipler nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede HSBC Türkiye icin mantikli pilot segmentini birlikte cikaralim.
+HSBC Türkiye bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: uluslararasi bankacilik ve global ekipler nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -893,14 +879,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K16" t="str">
-        <x:v>Merhaba Lütfü, Albaraka Türk icin İnsan ve Kültür Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda katilim bankaciligi ve surdurulebilirlik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'katilim bankaciligi ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Lütfü, Albaraka Türk için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L16" t="str">
-        <x:v>Subject: Albaraka Türk ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Albaraka Türk için 2 haftalık İngilizce gelişim pilotu
 Merhaba Lütfü,
-Albaraka Türk ekibinin Banking / Finance olceginde katilim bankaciligi ve surdurulebilirlik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: katilim bankaciligi ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Albaraka Türk icin mantikli pilot segmentini birlikte cikaralim.
+Albaraka Türk liderlik ekibinde İnsan ve Kültür Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -938,14 +923,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K17" t="str">
-        <x:v>Merhaba Bike, Alternatif Bank icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda ticari bankacilik ve yenilikci urunler nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'ticari bankacilik ve yenilikci urunler nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Bike, Alternatif Bank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L17" t="str">
-        <x:v>Subject: Alternatif Bank ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Alternatif Bank organizasyonel İngilizce gelişim standardı
 Merhaba Bike,
-Alternatif Bank ekibinin Banking / Finance olceginde ticari bankacilik ve yenilikci urunler odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: ticari bankacilik ve yenilikci urunler nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Alternatif Bank icin mantikli pilot segmentini birlikte cikaralim.
+Alternatif Bank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: ticari bankacilik ve yenilikci urunler nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -983,14 +967,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K18" t="str">
-        <x:v>Merhaba Beti, Trendyol icin İnsan Kaynakları Başkanı (CHRO) rolunuzu gordum. E-commerce / Marketplace tarafinda hizli olceklenen ekipler ve uluslararasi operasyon nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'hizli olceklenen ekipler ve uluslararasi operasyon nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Beti, Trendyol için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L18" t="str">
-        <x:v>Subject: Trendyol ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Trendyol için 2 haftalık İngilizce gelişim pilotu
 Merhaba Beti,
-Trendyol ekibinin E-commerce / Marketplace olceginde hizli olceklenen ekipler ve uluslararasi operasyon odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: hizli olceklenen ekipler ve uluslararasi operasyon nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Trendyol icin mantikli pilot segmentini birlikte cikaralim.
+Trendyol liderlik ekibinde İnsan Kaynakları Başkanı (CHRO) olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1028,14 +1011,13 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K19" t="str">
-        <x:v>Merhaba Tuğçe, Trendyol icin People and Culture Leader rolunuzu gordum. E-commerce / Marketplace tarafinda hizli olceklenen ekipler ve uluslararasi operasyon nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Tuğçe, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L19" t="str">
-        <x:v>Subject: Trendyol ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Trendyol çalışan bağlılığı ve kişisel gelişim fırsatları
 Merhaba Tuğçe,
-Trendyol ekibinin E-commerce / Marketplace olceginde hizli olceklenen ekipler ve uluslararasi operasyon odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Trendyol icin mantikli pilot segmentini birlikte cikaralim.
+Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1073,14 +1055,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K20" t="str">
-        <x:v>Merhaba Esra, Hepsiburada icin İnsan Kaynakları Grup Başkanı rolunuzu gordum. E-commerce / Marketplace tarafinda e-ticaret buyumesi ve teknoloji yatirimlari nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'e-ticaret buyumesi ve teknoloji yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Esra, Hepsiburada için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L20" t="str">
-        <x:v>Subject: Hepsiburada ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Hepsiburada için 2 haftalık İngilizce gelişim pilotu
 Merhaba Esra,
-Hepsiburada ekibinin E-commerce / Marketplace olceginde e-ticaret buyumesi ve teknoloji yatirimlari odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: e-ticaret buyumesi ve teknoloji yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Hepsiburada icin mantikli pilot segmentini birlikte cikaralim.
+Hepsiburada liderlik ekibinde İnsan Kaynakları Grup Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1118,14 +1099,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K21" t="str">
-        <x:v>Merhaba Petek, Getir icin İnsandan Sorumlu Genel Müdür Yardımcısı rolunuzu gordum. Quick commerce / Delivery tarafinda cok lokasyonlu operasyon ve saha ekipleri nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'cok lokasyonlu operasyon ve saha ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Petek, Getir genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L21" t="str">
-        <x:v>Subject: Getir ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Getir organizasyonel İngilizce gelişim standardı
 Merhaba Petek,
-Getir ekibinin Quick commerce / Delivery olceginde cok lokasyonlu operasyon ve saha ekipleri odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: cok lokasyonlu operasyon ve saha ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Getir icin mantikli pilot segmentini birlikte cikaralim.
+Getir bünyesinde Quick commerce / Delivery ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: cok lokasyonlu operasyon ve saha ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1163,14 +1143,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K22" t="str">
-        <x:v>Merhaba Alev, Dream Games icin HR Director rolunuzu gordum. Gaming / Technology tarafinda global urun ekipleri ve hizli ise alim nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global urun ekipleri ve hizli ise alim nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Alev, Dream Games için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L22" t="str">
-        <x:v>Subject: Dream Games ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Dream Games için 2 haftalık İngilizce gelişim pilotu
 Merhaba Alev,
-Dream Games ekibinin Gaming / Technology olceginde global urun ekipleri ve hizli ise alim odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global urun ekipleri ve hizli ise alim nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Dream Games icin mantikli pilot segmentini birlikte cikaralim.
+Dream Games liderlik ekibinde HR Director olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1208,14 +1187,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K23" t="str">
-        <x:v>Merhaba Eda, Peak Games icin İnsan Kaynakları Direktörü rolunuzu gordum. Gaming / Technology tarafinda global urun ve cok uluslu calisma ritmi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global urun ve cok uluslu calisma ritmi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Eda, Peak Games genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L23" t="str">
-        <x:v>Subject: Peak Games ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Peak Games organizasyonel İngilizce gelişim standardı
 Merhaba Eda,
-Peak Games ekibinin Gaming / Technology olceginde global urun ve cok uluslu calisma ritmi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global urun ve cok uluslu calisma ritmi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Peak Games icin mantikli pilot segmentini birlikte cikaralim.
+Peak Games bünyesinde Gaming / Technology ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global urun ve cok uluslu calisma ritmi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1253,14 +1231,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K24" t="str">
-        <x:v>Merhaba Nebahat, Logo Yazılım icin Grup İnsan ve Organizasyonel Dönüşüm Direktörü rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Nebahat, Logo Yazılım için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L24" t="str">
-        <x:v>Subject: Logo Yazılım ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Logo Yazılım için 2 haftalık İngilizce gelişim pilotu
 Merhaba Nebahat,
-Logo Yazılım ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Logo Yazılım icin mantikli pilot segmentini birlikte cikaralim.
+Logo Yazılım liderlik ekibinde Grup İnsan ve Organizasyonel Dönüşüm Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1298,14 +1275,13 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K25" t="str">
-        <x:v>Merhaba Aşkın, Yemeksepeti icin Head of People rolunuzu gordum. Food delivery / Tech tarafinda operasyon, satis ve teknoloji ekipleri nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Aşkın, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L25" t="str">
-        <x:v>Subject: Yemeksepeti ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Yemeksepeti çalışan bağlılığı ve kişisel gelişim fırsatları
 Merhaba Aşkın,
-Yemeksepeti ekibinin Food delivery / Tech olceginde operasyon, satis ve teknoloji ekipleri odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Yemeksepeti icin mantikli pilot segmentini birlikte cikaralim.
+Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1343,14 +1319,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K26" t="str">
-        <x:v>Merhaba Güntülü, Sahibinden.com icin İnsan ve Sürdürülebilirlik Genel Müdür Yardımcısı rolunuzu gordum. Classifieds / Technology tarafinda dijital pazar yeri ve teknoloji ekipleri nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'dijital pazar yeri ve teknoloji ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Güntülü, Sahibinden.com için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L26" t="str">
-        <x:v>Subject: Sahibinden.com ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Sahibinden.com için 2 haftalık İngilizce gelişim pilotu
 Merhaba Güntülü,
-Sahibinden.com ekibinin Classifieds / Technology olceginde dijital pazar yeri ve teknoloji ekipleri odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: dijital pazar yeri ve teknoloji ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Sahibinden.com icin mantikli pilot segmentini birlikte cikaralim.
+Sahibinden.com liderlik ekibinde İnsan ve Sürdürülebilirlik Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1388,14 +1363,13 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K27" t="str">
-        <x:v>Merhaba Gözde, BiTaksi icin Head of People rolunuzu gordum. Mobility / Technology tarafinda ulasim teknolojisi ve operasyon ekipleri nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Gözde, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L27" t="str">
-        <x:v>Subject: BiTaksi ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: BiTaksi çalışan bağlılığı ve kişisel gelişim fırsatları
 Merhaba Gözde,
-BiTaksi ekibinin Mobility / Technology olceginde ulasim teknolojisi ve operasyon ekipleri odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede BiTaksi icin mantikli pilot segmentini birlikte cikaralim.
+Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1433,14 +1407,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K28" t="str">
-        <x:v>Merhaba Tolga, Colendi icin HR Advisor to CEO rolunuzu gordum. Fintech tarafinda uluslararasi fintech urunlesmesi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'uluslararasi fintech urunlesmesi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Tolga, Colendi için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L28" t="str">
-        <x:v>Subject: Colendi ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Colendi için 2 haftalık İngilizce gelişim pilotu
 Merhaba Tolga,
-Colendi ekibinin Fintech olceginde uluslararasi fintech urunlesmesi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: uluslararasi fintech urunlesmesi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Colendi icin mantikli pilot segmentini birlikte cikaralim.
+Colendi liderlik ekibinde HR Advisor to CEO olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1478,14 +1451,13 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K29" t="str">
-        <x:v>Merhaba Dilara, Papara icin Senior People Partner rolunuzu gordum. Fintech tarafinda fintech buyumesi ve regulasyonla uyumlu ekipler nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Dilara, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L29" t="str">
-        <x:v>Subject: Papara ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Papara çalışan bağlılığı ve kişisel gelişim fırsatları
 Merhaba Dilara,
-Papara ekibinin Fintech olceginde fintech buyumesi ve regulasyonla uyumlu ekipler odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Papara icin mantikli pilot segmentini birlikte cikaralim.
+Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1523,14 +1495,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K30" t="str">
-        <x:v>Merhaba Seda, AloTech icin CHRO rolunuzu gordum. B2B SaaS / Technology tarafinda musteri deneyimi teknolojisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'musteri deneyimi teknolojisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Seda, AloTech için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L30" t="str">
-        <x:v>Subject: AloTech ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: AloTech için 2 haftalık İngilizce gelişim pilotu
 Merhaba Seda,
-AloTech ekibinin B2B SaaS / Technology olceginde musteri deneyimi teknolojisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: musteri deneyimi teknolojisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede AloTech icin mantikli pilot segmentini birlikte cikaralim.
+AloTech liderlik ekibinde CHRO olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1568,14 +1539,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K31" t="str">
-        <x:v>Merhaba Murat, Papel icin CHRO rolunuzu gordum. Fintech tarafinda dijital odeme ve fintech buyumesi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'dijital odeme ve fintech buyumesi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Murat, Papel genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L31" t="str">
-        <x:v>Subject: Papel ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Papel organizasyonel İngilizce gelişim standardı
 Merhaba Murat,
-Papel ekibinin Fintech olceginde dijital odeme ve fintech buyumesi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: dijital odeme ve fintech buyumesi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Papel icin mantikli pilot segmentini birlikte cikaralim.
+Papel bünyesinde Fintech ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: dijital odeme ve fintech buyumesi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1613,14 +1583,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K32" t="str">
-        <x:v>Merhaba Selin, Bilyoner icin CHRO rolunuzu gordum. iGaming / Technology tarafinda dijital bahis ve teknoloji ekipleri nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'dijital bahis ve teknoloji ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Selin, Bilyoner için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L32" t="str">
-        <x:v>Subject: Bilyoner ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Bilyoner için 2 haftalık İngilizce gelişim pilotu
 Merhaba Selin,
-Bilyoner ekibinin iGaming / Technology olceginde dijital bahis ve teknoloji ekipleri odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: dijital bahis ve teknoloji ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Bilyoner icin mantikli pilot segmentini birlikte cikaralim.
+Bilyoner liderlik ekibinde CHRO olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1658,14 +1627,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K33" t="str">
-        <x:v>Merhaba Erkan, Turkcell icin İnsan ve İş Destekten Sorumlu Genel Müdür Yardımcısı rolunuzu gordum. Telecommunications tarafinda kurumsal donusum ve teknoloji yetkinlikleri nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'kurumsal donusum ve teknoloji yetkinlikleri nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Erkan, Turkcell genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L33" t="str">
-        <x:v>Subject: Turkcell ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Turkcell organizasyonel İngilizce gelişim standardı
 Merhaba Erkan,
-Turkcell ekibinin Telecommunications olceginde kurumsal donusum ve teknoloji yetkinlikleri odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: kurumsal donusum ve teknoloji yetkinlikleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Turkcell icin mantikli pilot segmentini birlikte cikaralim.
+Turkcell bünyesinde Telecommunications ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: kurumsal donusum ve teknoloji yetkinlikleri nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1703,14 +1671,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K34" t="str">
-        <x:v>Merhaba Nazlı, Vodafone Türkiye icin İnsan Kaynaklarından Sorumlu İcra Kurulu Başkan Yardımcısı rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Nazlı, Vodafone Türkiye için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L34" t="str">
-        <x:v>Subject: Vodafone Türkiye ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Vodafone Türkiye için 2 haftalık İngilizce gelişim pilotu
 Merhaba Nazlı,
-Vodafone Türkiye ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Vodafone Türkiye icin mantikli pilot segmentini birlikte cikaralim.
+Vodafone Türkiye liderlik ekibinde İnsan Kaynaklarından Sorumlu İcra Kurulu Başkan Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1748,14 +1715,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K35" t="str">
-        <x:v>Merhaba İskender, Türk Telekom icin İnsan Kaynakları Genel Müdür Yardımcısı (CHRO) rolunuzu gordum. Telecommunications tarafinda dijital donusum ve fiber altyapi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'dijital donusum ve fiber altyapi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam İskender, Türk Telekom genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L35" t="str">
-        <x:v>Subject: Türk Telekom ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Türk Telekom organizasyonel İngilizce gelişim standardı
 Merhaba İskender,
-Türk Telekom ekibinin Telecommunications olceginde dijital donusum ve fiber altyapi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: dijital donusum ve fiber altyapi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Türk Telekom icin mantikli pilot segmentini birlikte cikaralim.
+Türk Telekom bünyesinde Telecommunications ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: dijital donusum ve fiber altyapi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1793,14 +1759,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K36" t="str">
-        <x:v>Merhaba Bahattin, LC Waikiki icin İnsan Kaynakları Genel Müdürü (CHRO) rolunuzu gordum. Retail / Fashion tarafinda magaza merkez ve yurt disi perakende operasyonlari nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'magaza merkez ve yurt disi perakende operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Bahattin, LC Waikiki için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L36" t="str">
-        <x:v>Subject: LC Waikiki ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: LC Waikiki için 2 haftalık İngilizce gelişim pilotu
 Merhaba Bahattin,
-LC Waikiki ekibinin Retail / Fashion olceginde magaza merkez ve yurt disi perakende operasyonlari odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: magaza merkez ve yurt disi perakende operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede LC Waikiki icin mantikli pilot segmentini birlikte cikaralim.
+LC Waikiki liderlik ekibinde İnsan Kaynakları Genel Müdürü (CHRO) olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1838,14 +1803,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K37" t="str">
-        <x:v>Merhaba Can, Mavi icin Chief Human Resources Officer (CHRO) rolunuzu gordum. Retail / Fashion tarafinda perakende ekipleri ve marka is birlikleri nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'perakende ekipleri ve marka is birlikleri nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Can, Mavi genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L37" t="str">
-        <x:v>Subject: Mavi ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Mavi organizasyonel İngilizce gelişim standardı
 Merhaba Can,
-Mavi ekibinin Retail / Fashion olceginde perakende ekipleri ve marka is birlikleri odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: perakende ekipleri ve marka is birlikleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Mavi icin mantikli pilot segmentini birlikte cikaralim.
+Mavi bünyesinde Retail / Fashion ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: perakende ekipleri ve marka is birlikleri nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1883,14 +1847,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K38" t="str">
-        <x:v>Merhaba Yeşim, DeFacto icin İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı rolunuzu gordum. Retail / Fashion tarafinda hizli moda ve uluslararasi buyume nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Yeşim, DeFacto için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L38" t="str">
-        <x:v>Subject: DeFacto ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: DeFacto için 2 haftalık İngilizce gelişim pilotu
 Merhaba Yeşim,
-DeFacto ekibinin Retail / Fashion olceginde hizli moda ve uluslararasi buyume odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede DeFacto icin mantikli pilot segmentini birlikte cikaralim.
+DeFacto liderlik ekibinde İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1928,14 +1891,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K39" t="str">
-        <x:v>Merhaba Yasemin, Boyner Grup icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Retail / Department store tarafinda cok kanalli perakende donusumu nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'cok kanalli perakende donusumu nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Yasemin, Boyner Grup genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L39" t="str">
-        <x:v>Subject: Boyner Grup ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Boyner Grup organizasyonel İngilizce gelişim standardı
 Merhaba Yasemin,
-Boyner Grup ekibinin Retail / Department store olceginde cok kanalli perakende donusumu odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: cok kanalli perakende donusumu nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Boyner Grup icin mantikli pilot segmentini birlikte cikaralim.
+Boyner Grup bünyesinde Retail / Department store ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: cok kanalli perakende donusumu nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1973,14 +1935,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K40" t="str">
-        <x:v>Merhaba Hasan, BİM icin İnsan Kaynakları Başkanı (CHRO) rolunuzu gordum. Retail / Discount tarafinda indirim perakende ve operasyonel verimlilik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'indirim perakende ve operasyonel verimlilik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Hasan, BİM için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L40" t="str">
-        <x:v>Subject: BİM ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: BİM için 2 haftalık İngilizce gelişim pilotu
 Merhaba Hasan,
-BİM ekibinin Retail / Discount olceginde indirim perakende ve operasyonel verimlilik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: indirim perakende ve operasyonel verimlilik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede BİM icin mantikli pilot segmentini birlikte cikaralim.
+BİM liderlik ekibinde İnsan Kaynakları Başkanı (CHRO) olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2018,14 +1979,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K41" t="str">
-        <x:v>Merhaba Olcay, Migros icin İnsan Kaynakları ve Endüstri İlişkileri GMY rolunuzu gordum. Retail / Grocery tarafinda gida perakende ve dijital donusum nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'gida perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Olcay, Migros genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L41" t="str">
-        <x:v>Subject: Migros ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Migros organizasyonel İngilizce gelişim standardı
 Merhaba Olcay,
-Migros ekibinin Retail / Grocery olceginde gida perakende ve dijital donusum odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: gida perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Migros icin mantikli pilot segmentini birlikte cikaralim.
+Migros bünyesinde Retail / Grocery ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: gida perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2063,14 +2023,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K42" t="str">
-        <x:v>Merhaba Bahar, CarrefourSA icin İnsan Kaynakları ve Sürdürülebilirlik GMY rolunuzu gordum. Retail / Grocery tarafinda gida perakende ve surdurulebilirlik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'gida perakende ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Bahar, CarrefourSA için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L42" t="str">
-        <x:v>Subject: CarrefourSA ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: CarrefourSA için 2 haftalık İngilizce gelişim pilotu
 Merhaba Bahar,
-CarrefourSA ekibinin Retail / Grocery olceginde gida perakende ve surdurulebilirlik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: gida perakende ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede CarrefourSA icin mantikli pilot segmentini birlikte cikaralim.
+CarrefourSA liderlik ekibinde İnsan Kaynakları ve Sürdürülebilirlik GMY olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2108,14 +2067,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K43" t="str">
-        <x:v>Merhaba Tuncer, ŞOK Marketler icin İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı rolunuzu gordum. Retail / Discount tarafinda hizli buyuyen indirim perakende nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'hizli buyuyen indirim perakende nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Tuncer, ŞOK Marketler genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L43" t="str">
-        <x:v>Subject: ŞOK Marketler ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: ŞOK Marketler organizasyonel İngilizce gelişim standardı
 Merhaba Tuncer,
-ŞOK Marketler ekibinin Retail / Discount olceginde hizli buyuyen indirim perakende odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: hizli buyuyen indirim perakende nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede ŞOK Marketler icin mantikli pilot segmentini birlikte cikaralim.
+ŞOK Marketler bünyesinde Retail / Discount ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: hizli buyuyen indirim perakende nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2153,14 +2111,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K44" t="str">
-        <x:v>Merhaba Eriş, Koçtaş icin İnsan Kaynakları ve Endüstri İlişkileri GMY rolunuzu gordum. Retail / Home improvement tarafinda yapi market ve perakende operasyonlari nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'yapi market ve perakende operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Eriş, Koçtaş için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L44" t="str">
-        <x:v>Subject: Koçtaş ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Koçtaş için 2 haftalık İngilizce gelişim pilotu
 Merhaba Eriş,
-Koçtaş ekibinin Retail / Home improvement olceginde yapi market ve perakende operasyonlari odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: yapi market ve perakende operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Koçtaş icin mantikli pilot segmentini birlikte cikaralim.
+Koçtaş liderlik ekibinde İnsan Kaynakları ve Endüstri İlişkileri GMY olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2198,14 +2155,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K45" t="str">
-        <x:v>Merhaba Ali, Ford Otosan icin İnsan Kaynakları Direktörü rolunuzu gordum. Automotive / Manufacturing tarafinda uretim, muhendislik ve global tedarik zinciri nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'uretim, muhendislik ve global tedarik zinciri nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Ali, Ford Otosan genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L45" t="str">
-        <x:v>Subject: Ford Otosan ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Ford Otosan organizasyonel İngilizce gelişim standardı
 Merhaba Ali,
-Ford Otosan ekibinin Automotive / Manufacturing olceginde uretim, muhendislik ve global tedarik zinciri odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: uretim, muhendislik ve global tedarik zinciri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Ford Otosan icin mantikli pilot segmentini birlikte cikaralim.
+Ford Otosan bünyesinde Automotive / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: uretim, muhendislik ve global tedarik zinciri nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2243,14 +2199,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K46" t="str">
-        <x:v>Merhaba Orçun, TOFAŞ icin İnsan Kaynakları ve Endüstriyel İlişkiler Direktörü rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Orçun, TOFAŞ için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L46" t="str">
-        <x:v>Subject: TOFAŞ ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: TOFAŞ için 2 haftalık İngilizce gelişim pilotu
 Merhaba Orçun,
-TOFAŞ ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede TOFAŞ icin mantikli pilot segmentini birlikte cikaralim.
+TOFAŞ liderlik ekibinde İnsan Kaynakları ve Endüstriyel İlişkiler Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2288,14 +2243,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K47" t="str">
-        <x:v>Merhaba Seda, Toyota Türkiye icin İnsan Kaynakları ve Tesis Yönetim Direktörü rolunuzu gordum. Automotive / Manufacturing tarafinda uretim ve kalite muhendisligi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'uretim ve kalite muhendisligi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Seda, Toyota Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L47" t="str">
-        <x:v>Subject: Toyota Türkiye ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Toyota Türkiye organizasyonel İngilizce gelişim standardı
 Merhaba Seda,
-Toyota Türkiye ekibinin Automotive / Manufacturing olceginde uretim ve kalite muhendisligi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: uretim ve kalite muhendisligi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Toyota Türkiye icin mantikli pilot segmentini birlikte cikaralim.
+Toyota Türkiye bünyesinde Automotive / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: uretim ve kalite muhendisligi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2333,14 +2287,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K48" t="str">
-        <x:v>Merhaba Betül, Mercedes-Benz Türk icin İnsan Kaynakları Direktörü rolunuzu gordum. Automotive / Manufacturing tarafinda premium otomotiv ve global standartlar nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'premium otomotiv ve global standartlar nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Betül, Mercedes-Benz Türk için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L48" t="str">
-        <x:v>Subject: Mercedes-Benz Türk ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Mercedes-Benz Türk için 2 haftalık İngilizce gelişim pilotu
 Merhaba Betül,
-Mercedes-Benz Türk ekibinin Automotive / Manufacturing olceginde premium otomotiv ve global standartlar odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: premium otomotiv ve global standartlar nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Mercedes-Benz Türk icin mantikli pilot segmentini birlikte cikaralim.
+Mercedes-Benz Türk liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2378,14 +2331,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K49" t="str">
-        <x:v>Merhaba Gökhan, Hyundai Assan icin İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı rolunuzu gordum. Automotive / Manufacturing tarafinda otomotiv uretim ve ihracat nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Gökhan, Hyundai Assan genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L49" t="str">
-        <x:v>Subject: Hyundai Assan ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Hyundai Assan organizasyonel İngilizce gelişim standardı
 Merhaba Gökhan,
-Hyundai Assan ekibinin Automotive / Manufacturing olceginde otomotiv uretim ve ihracat odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Hyundai Assan icin mantikli pilot segmentini birlikte cikaralim.
+Hyundai Assan bünyesinde Automotive / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2423,14 +2375,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K50" t="str">
-        <x:v>Merhaba Dr., Renault MAİS icin İnsan Kaynakları Direktörü rolunuzu gordum. Automotive / Distribution tarafinda otomotiv dagitim ve satis nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'otomotiv dagitim ve satis nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Dr., Renault MAİS için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L50" t="str">
-        <x:v>Subject: Renault MAİS ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Renault MAİS için 2 haftalık İngilizce gelişim pilotu
 Merhaba Dr.,
-Renault MAİS ekibinin Automotive / Distribution olceginde otomotiv dagitim ve satis odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: otomotiv dagitim ve satis nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Renault MAİS icin mantikli pilot segmentini birlikte cikaralim.
+Renault MAİS liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2468,14 +2419,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K51" t="str">
-        <x:v>Merhaba Fikri, Arçelik icin Kıdemli Direktör, İnsan Kaynakları rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Fikri, Arçelik genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L51" t="str">
-        <x:v>Subject: Arçelik ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Arçelik organizasyonel İngilizce gelişim standardı
 Merhaba Fikri,
-Arçelik ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Arçelik icin mantikli pilot segmentini birlikte cikaralim.
+Arçelik bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2513,14 +2463,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K52" t="str">
-        <x:v>Merhaba Zeynep, Vestel icin İnsan Kaynakları Genel Müdürü rolunuzu gordum. Electronics / Manufacturing tarafinda ihracat agi ve teknik ekiplerin Ingilizce ihtiyaci nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'ihracat agi ve teknik ekiplerin Ingilizce ihtiyaci nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Zeynep, Vestel için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L52" t="str">
-        <x:v>Subject: Vestel ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Vestel için 2 haftalık İngilizce gelişim pilotu
 Merhaba Zeynep,
-Vestel ekibinin Electronics / Manufacturing olceginde ihracat agi ve teknik ekiplerin Ingilizce ihtiyaci odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: ihracat agi ve teknik ekiplerin Ingilizce ihtiyaci nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Vestel icin mantikli pilot segmentini birlikte cikaralim.
+Vestel liderlik ekibinde İnsan Kaynakları Genel Müdürü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2558,14 +2507,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K53" t="str">
-        <x:v>Merhaba Nursel, Borusan Holding icin İnsan Kaynakları ve Kurumsal İletişim Grup Başkanı rolunuzu gordum. Conglomerate / Industrial tarafinda sanayi ve hizmet sektoru yonetimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'sanayi ve hizmet sektoru yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Nursel, Borusan Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L53" t="str">
-        <x:v>Subject: Borusan Holding ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Borusan Holding organizasyonel İngilizce gelişim standardı
 Merhaba Nursel,
-Borusan Holding ekibinin Conglomerate / Industrial olceginde sanayi ve hizmet sektoru yonetimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: sanayi ve hizmet sektoru yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Borusan Holding icin mantikli pilot segmentini birlikte cikaralim.
+Borusan Holding bünyesinde Conglomerate / Industrial ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: sanayi ve hizmet sektoru yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2603,14 +2551,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K54" t="str">
-        <x:v>Merhaba Tuğba, Borusan Otomotiv icin İK ve İSG'den Sorumlu İcra Kurulu Üyesi rolunuzu gordum. Automotive / Distribution tarafinda premium otomotiv dagitim nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'premium otomotiv dagitim nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Tuğba, Borusan Otomotiv için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L54" t="str">
-        <x:v>Subject: Borusan Otomotiv ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Borusan Otomotiv için 2 haftalık İngilizce gelişim pilotu
 Merhaba Tuğba,
-Borusan Otomotiv ekibinin Automotive / Distribution olceginde premium otomotiv dagitim odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: premium otomotiv dagitim nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Borusan Otomotiv icin mantikli pilot segmentini birlikte cikaralim.
+Borusan Otomotiv liderlik ekibinde İK ve İSG'den Sorumlu İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2648,14 +2595,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K55" t="str">
-        <x:v>Merhaba Şengül, Şişecam icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Glass / Manufacturing tarafinda cam sanayi ve global operasyonlar nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'cam sanayi ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Şengül, Şişecam genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L55" t="str">
-        <x:v>Subject: Şişecam ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Şişecam organizasyonel İngilizce gelişim standardı
 Merhaba Şengül,
-Şişecam ekibinin Glass / Manufacturing olceginde cam sanayi ve global operasyonlar odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: cam sanayi ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Şişecam icin mantikli pilot segmentini birlikte cikaralim.
+Şişecam bünyesinde Glass / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: cam sanayi ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2693,14 +2639,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K56" t="str">
-        <x:v>Merhaba Neslihan, Kordsa icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Industrial / Manufacturing tarafinda endüstriyel tekstil ve global uretim nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'endüstriyel tekstil ve global uretim nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Neslihan, Kordsa için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L56" t="str">
-        <x:v>Subject: Kordsa ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Kordsa için 2 haftalık İngilizce gelişim pilotu
 Merhaba Neslihan,
-Kordsa ekibinin Industrial / Manufacturing olceginde endüstriyel tekstil ve global uretim odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: endüstriyel tekstil ve global uretim nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Kordsa icin mantikli pilot segmentini birlikte cikaralim.
+Kordsa liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2738,14 +2683,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K57" t="str">
-        <x:v>Merhaba Tuğba, Brisa icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Tire / Manufacturing tarafinda lastik uretimi ve Bridgestone is birligi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'lastik uretimi ve Bridgestone is birligi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Tuğba, Brisa genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L57" t="str">
-        <x:v>Subject: Brisa ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Brisa organizasyonel İngilizce gelişim standardı
 Merhaba Tuğba,
-Brisa ekibinin Tire / Manufacturing olceginde lastik uretimi ve Bridgestone is birligi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: lastik uretimi ve Bridgestone is birligi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Brisa icin mantikli pilot segmentini birlikte cikaralim.
+Brisa bünyesinde Tire / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: lastik uretimi ve Bridgestone is birligi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2783,14 +2727,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K58" t="str">
-        <x:v>Merhaba Tuncay, Doğan Holding icin İnsan Kaynakları Direktörü rolunuzu gordum. Conglomerate / Media tarafinda medya enerji ve sanayi yonetimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'medya enerji ve sanayi yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Tuncay, Doğan Holding için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L58" t="str">
-        <x:v>Subject: Doğan Holding ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Doğan Holding için 2 haftalık İngilizce gelişim pilotu
 Merhaba Tuncay,
-Doğan Holding ekibinin Conglomerate / Media olceginde medya enerji ve sanayi yonetimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: medya enerji ve sanayi yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Doğan Holding icin mantikli pilot segmentini birlikte cikaralim.
+Doğan Holding liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2828,14 +2771,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K59" t="str">
-        <x:v>Merhaba Abdulkerim, Türk Hava Yolları icin İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı rolunuzu gordum. Airlines / Aviation tarafinda global havayolu ve genis operasyon agi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global havayolu ve genis operasyon agi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Abdulkerim, Türk Hava Yolları genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L59" t="str">
-        <x:v>Subject: Türk Hava Yolları ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Türk Hava Yolları organizasyonel İngilizce gelişim standardı
 Merhaba Abdulkerim,
-Türk Hava Yolları ekibinin Airlines / Aviation olceginde global havayolu ve genis operasyon agi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global havayolu ve genis operasyon agi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Türk Hava Yolları icin mantikli pilot segmentini birlikte cikaralim.
+Türk Hava Yolları bünyesinde Airlines / Aviation ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global havayolu ve genis operasyon agi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2873,14 +2815,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K60" t="str">
-        <x:v>Merhaba Dilara, Pegasus Hava Yolları icin İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı rolunuzu gordum. Airlines / Aviation tarafinda dusuk maliyet havayolu ve hizli buyume nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'dusuk maliyet havayolu ve hizli buyume nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Dilara, Pegasus Hava Yolları için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L60" t="str">
-        <x:v>Subject: Pegasus Hava Yolları ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Pegasus Hava Yolları için 2 haftalık İngilizce gelişim pilotu
 Merhaba Dilara,
-Pegasus Hava Yolları ekibinin Airlines / Aviation olceginde dusuk maliyet havayolu ve hizli buyume odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: dusuk maliyet havayolu ve hizli buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Pegasus Hava Yolları icin mantikli pilot segmentini birlikte cikaralim.
+Pegasus Hava Yolları liderlik ekibinde İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2918,14 +2859,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K61" t="str">
-        <x:v>Merhaba Berrin, Enerjisa icin İnsan ve Kültür Bölüm Başkanı (CHRO) rolunuzu gordum. Energy / Utilities tarafinda enerji dagitim ve surdurulebilirlik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'enerji dagitim ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Berrin, Enerjisa genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L61" t="str">
-        <x:v>Subject: Enerjisa ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Enerjisa organizasyonel İngilizce gelişim standardı
 Merhaba Berrin,
-Enerjisa ekibinin Energy / Utilities olceginde enerji dagitim ve surdurulebilirlik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: enerji dagitim ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Enerjisa icin mantikli pilot segmentini birlikte cikaralim.
+Enerjisa bünyesinde Energy / Utilities ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: enerji dagitim ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2963,14 +2903,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K62" t="str">
-        <x:v>Merhaba Önder, TÜPRAŞ icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Energy / Refining tarafinda rafineri ve petrokimya uretimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'rafineri ve petrokimya uretimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Önder, TÜPRAŞ için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L62" t="str">
-        <x:v>Subject: TÜPRAŞ ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: TÜPRAŞ için 2 haftalık İngilizce gelişim pilotu
 Merhaba Önder,
-TÜPRAŞ ekibinin Energy / Refining olceginde rafineri ve petrokimya uretimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: rafineri ve petrokimya uretimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede TÜPRAŞ icin mantikli pilot segmentini birlikte cikaralim.
+TÜPRAŞ liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3008,14 +2947,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K63" t="str">
-        <x:v>Merhaba Gülay, Aksa Enerji icin İnsan Kaynakları Direktörü rolunuzu gordum. Energy / Power tarafinda enerji uretim ve yatirimlari nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'enerji uretim ve yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Gülay, Aksa Enerji genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L63" t="str">
-        <x:v>Subject: Aksa Enerji ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Aksa Enerji organizasyonel İngilizce gelişim standardı
 Merhaba Gülay,
-Aksa Enerji ekibinin Energy / Power olceginde enerji uretim ve yatirimlari odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: enerji uretim ve yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Aksa Enerji icin mantikli pilot segmentini birlikte cikaralim.
+Aksa Enerji bünyesinde Energy / Power ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: enerji uretim ve yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3053,14 +2991,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K64" t="str">
-        <x:v>Merhaba Burcu, Unilever Türkiye icin İnsan Kaynakları Başkanı rolunuzu gordum. FMCG / Consumer goods tarafinda global FMCG ve cok uluslu calisma nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global FMCG ve cok uluslu calisma nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Burcu, Unilever Türkiye için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L64" t="str">
-        <x:v>Subject: Unilever Türkiye ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Unilever Türkiye için 2 haftalık İngilizce gelişim pilotu
 Merhaba Burcu,
-Unilever Türkiye ekibinin FMCG / Consumer goods olceginde global FMCG ve cok uluslu calisma odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global FMCG ve cok uluslu calisma nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Unilever Türkiye icin mantikli pilot segmentini birlikte cikaralim.
+Unilever Türkiye liderlik ekibinde İnsan Kaynakları Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3098,14 +3035,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K65" t="str">
-        <x:v>Merhaba Mısra, P&amp;G Türkiye icin Kıdemli İnsan Kaynakları Direktörü rolunuzu gordum. FMCG / Consumer goods tarafinda global standartlar ve liderlik gelisimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global standartlar ve liderlik gelisimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Mısra, P&amp;G Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L65" t="str">
-        <x:v>Subject: P&amp;G Türkiye ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: P&amp;G Türkiye organizasyonel İngilizce gelişim standardı
 Merhaba Mısra,
-P&amp;G Türkiye ekibinin FMCG / Consumer goods olceginde global standartlar ve liderlik gelisimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global standartlar ve liderlik gelisimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede P&amp;G Türkiye icin mantikli pilot segmentini birlikte cikaralim.
+P&amp;G Türkiye bünyesinde FMCG / Consumer goods ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global standartlar ve liderlik gelisimi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3143,14 +3079,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K66" t="str">
-        <x:v>Merhaba Burak, Coca-Cola İçecek icin İnsan Kaynaklarından Sorumlu İcra Kurulu Üyesi rolunuzu gordum. Beverages / FMCG tarafinda global marka ve cok ulkeli operasyonlar nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global marka ve cok ulkeli operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Burak, Coca-Cola İçecek için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L66" t="str">
-        <x:v>Subject: Coca-Cola İçecek ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Coca-Cola İçecek için 2 haftalık İngilizce gelişim pilotu
 Merhaba Burak,
-Coca-Cola İçecek ekibinin Beverages / FMCG olceginde global marka ve cok ulkeli operasyonlar odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global marka ve cok ulkeli operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Coca-Cola İçecek icin mantikli pilot segmentini birlikte cikaralim.
+Coca-Cola İçecek liderlik ekibinde İnsan Kaynaklarından Sorumlu İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3188,14 +3123,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K67" t="str">
-        <x:v>Merhaba Oktay, Nestlé Türkiye icin İnsan Kaynakları Direktörü rolunuzu gordum. FMCG / Food tarafinda global gida sirketi ve surdurulebilirlik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global gida sirketi ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Oktay, Nestlé Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L67" t="str">
-        <x:v>Subject: Nestlé Türkiye ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Nestlé Türkiye organizasyonel İngilizce gelişim standardı
 Merhaba Oktay,
-Nestlé Türkiye ekibinin FMCG / Food olceginde global gida sirketi ve surdurulebilirlik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global gida sirketi ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Nestlé Türkiye icin mantikli pilot segmentini birlikte cikaralim.
+Nestlé Türkiye bünyesinde FMCG / Food ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global gida sirketi ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3233,14 +3167,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K68" t="str">
-        <x:v>Merhaba Oğuzhan, Anadolu Efes icin Türkiye İnsan Kaynakları Direktörü rolunuzu gordum. Beverages / FMCG tarafinda icecek sektoru ve uluslararasi operasyonlar nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'icecek sektoru ve uluslararasi operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Oğuzhan, Anadolu Efes için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L68" t="str">
-        <x:v>Subject: Anadolu Efes ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Anadolu Efes için 2 haftalık İngilizce gelişim pilotu
 Merhaba Oğuzhan,
-Anadolu Efes ekibinin Beverages / FMCG olceginde icecek sektoru ve uluslararasi operasyonlar odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: icecek sektoru ve uluslararasi operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Anadolu Efes icin mantikli pilot segmentini birlikte cikaralim.
+Anadolu Efes liderlik ekibinde Türkiye İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3278,14 +3211,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K69" t="str">
-        <x:v>Merhaba Eylem, Ülker / Yıldız Holding icin İnsan Kaynakları Başkan Yardımcısı rolunuzu gordum. FMCG / Food tarafinda gida uretimi ve global marka portfoyu nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'gida uretimi ve global marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Eylem, Ülker / Yıldız Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L69" t="str">
-        <x:v>Subject: Ülker / Yıldız Holding ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Ülker / Yıldız Holding organizasyonel İngilizce gelişim standardı
 Merhaba Eylem,
-Ülker / Yıldız Holding ekibinin FMCG / Food olceginde gida uretimi ve global marka portfoyu odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: gida uretimi ve global marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Ülker / Yıldız Holding icin mantikli pilot segmentini birlikte cikaralim.
+Ülker / Yıldız Holding bünyesinde FMCG / Food ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: gida uretimi ve global marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3323,14 +3255,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K70" t="str">
-        <x:v>Merhaba Umut, Koç Holding icin İnsan Kaynakları Direktörü rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Umut, Koç Holding için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L70" t="str">
-        <x:v>Subject: Koç Holding ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Koç Holding için 2 haftalık İngilizce gelişim pilotu
 Merhaba Umut,
-Koç Holding ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Koç Holding icin mantikli pilot segmentini birlikte cikaralim.
+Koç Holding liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3368,14 +3299,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K71" t="str">
-        <x:v>Merhaba Yeşim, Sabancı Holding icin İnsan Kaynakları ve Sürdürülebilirlik Grup Başkanı rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Yeşim, Sabancı Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L71" t="str">
-        <x:v>Subject: Sabancı Holding ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Sabancı Holding organizasyonel İngilizce gelişim standardı
 Merhaba Yeşim,
-Sabancı Holding ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Sabancı Holding icin mantikli pilot segmentini birlikte cikaralim.
+Sabancı Holding bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3413,14 +3343,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K72" t="str">
-        <x:v>Merhaba Hakan, Zorlu Holding icin İnsan Kaynakları Grubu Başkanı rolunuzu gordum. Conglomerate tarafinda enerji tekstil teknoloji ve gayrimenkul nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'enerji tekstil teknoloji ve gayrimenkul nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Hakan, Zorlu Holding için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L72" t="str">
-        <x:v>Subject: Zorlu Holding ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Zorlu Holding için 2 haftalık İngilizce gelişim pilotu
 Merhaba Hakan,
-Zorlu Holding ekibinin Conglomerate olceginde enerji tekstil teknoloji ve gayrimenkul odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: enerji tekstil teknoloji ve gayrimenkul nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Zorlu Holding icin mantikli pilot segmentini birlikte cikaralim.
+Zorlu Holding liderlik ekibinde İnsan Kaynakları Grubu Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3458,14 +3387,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K73" t="str">
-        <x:v>Merhaba Evrim, Eczacıbaşı Holding icin İnsan Kaynakları Grup Başkanı rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Evrim, Eczacıbaşı Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L73" t="str">
-        <x:v>Subject: Eczacıbaşı Holding ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Eczacıbaşı Holding organizasyonel İngilizce gelişim standardı
 Merhaba Evrim,
-Eczacıbaşı Holding ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Eczacıbaşı Holding icin mantikli pilot segmentini birlikte cikaralim.
+Eczacıbaşı Holding bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3503,14 +3431,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K74" t="str">
-        <x:v>Merhaba Özge, Kalyon Holding icin İnsan Kaynakları Grup Başkanı rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Özge, Kalyon Holding için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L74" t="str">
-        <x:v>Subject: Kalyon Holding ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Kalyon Holding için 2 haftalık İngilizce gelişim pilotu
 Merhaba Özge,
-Kalyon Holding ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Kalyon Holding icin mantikli pilot segmentini birlikte cikaralim.
+Kalyon Holding liderlik ekibinde İnsan Kaynakları Grup Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3548,14 +3475,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K75" t="str">
-        <x:v>Merhaba Melis, TAV Havalimanları icin İnsan Kaynakları Grup Başkanı (CHRO) rolunuzu gordum. Aviation / Infrastructure tarafinda havalimani isletme ve global operasyonlar nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'havalimani isletme ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Melis, TAV Havalimanları genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L75" t="str">
-        <x:v>Subject: TAV Havalimanları ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: TAV Havalimanları organizasyonel İngilizce gelişim standardı
 Merhaba Melis,
-TAV Havalimanları ekibinin Aviation / Infrastructure olceginde havalimani isletme ve global operasyonlar odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: havalimani isletme ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede TAV Havalimanları icin mantikli pilot segmentini birlikte cikaralim.
+TAV Havalimanları bünyesinde Aviation / Infrastructure ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: havalimani isletme ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3593,14 +3519,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K76" t="str">
-        <x:v>Merhaba Yalçın, Doğuş Otomotiv icin İnsan Kaynakları ve Süreç Yönetimi Direktörü rolunuzu gordum. Automotive / Distribution tarafinda otomotiv dagitim ve perakende nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'otomotiv dagitim ve perakende nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Yalçın, Doğuş Otomotiv için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L76" t="str">
-        <x:v>Subject: Doğuş Otomotiv ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Doğuş Otomotiv için 2 haftalık İngilizce gelişim pilotu
 Merhaba Yalçın,
-Doğuş Otomotiv ekibinin Automotive / Distribution olceginde otomotiv dagitim ve perakende odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: otomotiv dagitim ve perakende nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Doğuş Otomotiv icin mantikli pilot segmentini birlikte cikaralim.
+Doğuş Otomotiv liderlik ekibinde İnsan Kaynakları ve Süreç Yönetimi Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3638,14 +3563,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K77" t="str">
-        <x:v>Merhaba Dr., Abdi İbrahim icin İK, Kurumsal İletişim ve Sürdürülebilirlik Grup Başkanı rolunuzu gordum. Pharma / Healthcare tarafinda ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Dr., Abdi İbrahim genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L77" t="str">
-        <x:v>Subject: Abdi İbrahim ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Abdi İbrahim organizasyonel İngilizce gelişim standardı
 Merhaba Dr.,
-Abdi İbrahim ekibinin Pharma / Healthcare olceginde ilac sanayi ve uluslararasi buyume odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Abdi İbrahim icin mantikli pilot segmentini birlikte cikaralim.
+Abdi İbrahim bünyesinde Pharma / Healthcare ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3683,14 +3607,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K78" t="str">
-        <x:v>Merhaba Ayşe, Abdi İbrahim icin Uluslararası Pazarlar İnsan Kaynakları Direktörü rolunuzu gordum. Pharma / Healthcare tarafinda ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Ayşe, Abdi İbrahim için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L78" t="str">
-        <x:v>Subject: Abdi İbrahim ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Abdi İbrahim için 2 haftalık İngilizce gelişim pilotu
 Merhaba Ayşe,
-Abdi İbrahim ekibinin Pharma / Healthcare olceginde ilac sanayi ve uluslararasi buyume odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Abdi İbrahim icin mantikli pilot segmentini birlikte cikaralim.
+Abdi İbrahim liderlik ekibinde Uluslararası Pazarlar İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3728,14 +3651,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K79" t="str">
-        <x:v>Merhaba Kader, Eczacıbaşı Sağlık icin İnsan Kaynakları Direktörü rolunuzu gordum. Healthcare / Pharma tarafinda saglik urunleri ve ilac nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'saglik urunleri ve ilac nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Kader, Eczacıbaşı Sağlık genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L79" t="str">
-        <x:v>Subject: Eczacıbaşı Sağlık ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Eczacıbaşı Sağlık organizasyonel İngilizce gelişim standardı
 Merhaba Kader,
-Eczacıbaşı Sağlık ekibinin Healthcare / Pharma olceginde saglik urunleri ve ilac odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: saglik urunleri ve ilac nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Eczacıbaşı Sağlık icin mantikli pilot segmentini birlikte cikaralim.
+Eczacıbaşı Sağlık bünyesinde Healthcare / Pharma ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: saglik urunleri ve ilac nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3773,14 +3695,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K80" t="str">
-        <x:v>Merhaba Demet, Medicana Sağlık Grubu icin İnsan Kaynakları Grup Başkanı rolunuzu gordum. Healthcare / Hospitals tarafinda ozel saglik ve hastane yonetimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'ozel saglik ve hastane yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Demet, Medicana Sağlık Grubu için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L80" t="str">
-        <x:v>Subject: Medicana Sağlık Grubu ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Medicana Sağlık Grubu için 2 haftalık İngilizce gelişim pilotu
 Merhaba Demet,
-Medicana Sağlık Grubu ekibinin Healthcare / Hospitals olceginde ozel saglik ve hastane yonetimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: ozel saglik ve hastane yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Medicana Sağlık Grubu icin mantikli pilot segmentini birlikte cikaralim.
+Medicana Sağlık Grubu liderlik ekibinde İnsan Kaynakları Grup Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3818,14 +3739,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K81" t="str">
-        <x:v>Merhaba Gökben, Acıbadem Sağlık Grubu icin İnsan Kaynakları Direktör Vekili rolunuzu gordum. Healthcare / Hospitals tarafinda premium saglik hizmetleri nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'premium saglik hizmetleri nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Gökben, Acıbadem Sağlık Grubu genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L81" t="str">
-        <x:v>Subject: Acıbadem Sağlık Grubu ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Acıbadem Sağlık Grubu organizasyonel İngilizce gelişim standardı
 Merhaba Gökben,
-Acıbadem Sağlık Grubu ekibinin Healthcare / Hospitals olceginde premium saglik hizmetleri odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: premium saglik hizmetleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Acıbadem Sağlık Grubu icin mantikli pilot segmentini birlikte cikaralim.
+Acıbadem Sağlık Grubu bünyesinde Healthcare / Hospitals ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: premium saglik hizmetleri nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3863,14 +3783,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K82" t="str">
-        <x:v>Merhaba Muhammed, ASELSAN icin İnsan Kaynakları Direktörü rolunuzu gordum. Defense / Technology tarafinda savunma teknolojisi ve muhendislik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'savunma teknolojisi ve muhendislik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Muhammed, ASELSAN için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L82" t="str">
-        <x:v>Subject: ASELSAN ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: ASELSAN için 2 haftalık İngilizce gelişim pilotu
 Merhaba Muhammed,
-ASELSAN ekibinin Defense / Technology olceginde savunma teknolojisi ve muhendislik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: savunma teknolojisi ve muhendislik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede ASELSAN icin mantikli pilot segmentini birlikte cikaralim.
+ASELSAN liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3908,14 +3827,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K83" t="str">
-        <x:v>Merhaba Oğuzhan, HAVELSAN icin İnsan Kaynakları Direktörü rolunuzu gordum. Defense / Technology tarafinda savunma yazilimi ve siber guvenlik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'savunma yazilimi ve siber guvenlik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Oğuzhan, HAVELSAN genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L83" t="str">
-        <x:v>Subject: HAVELSAN ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: HAVELSAN organizasyonel İngilizce gelişim standardı
 Merhaba Oğuzhan,
-HAVELSAN ekibinin Defense / Technology olceginde savunma yazilimi ve siber guvenlik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: savunma yazilimi ve siber guvenlik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede HAVELSAN icin mantikli pilot segmentini birlikte cikaralim.
+HAVELSAN bünyesinde Defense / Technology ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: savunma yazilimi ve siber guvenlik nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3953,14 +3871,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K84" t="str">
-        <x:v>Merhaba Zeynep, AXA Sigorta icin İnsan Kaynakları Direktörü ve İcra Kurulu Üyesi rolunuzu gordum. Insurance / Finance tarafinda global sigorta ve risk yonetimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global sigorta ve risk yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Zeynep, AXA Sigorta için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L84" t="str">
-        <x:v>Subject: AXA Sigorta ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: AXA Sigorta için 2 haftalık İngilizce gelişim pilotu
 Merhaba Zeynep,
-AXA Sigorta ekibinin Insurance / Finance olceginde global sigorta ve risk yonetimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global sigorta ve risk yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede AXA Sigorta icin mantikli pilot segmentini birlikte cikaralim.
+AXA Sigorta liderlik ekibinde İnsan Kaynakları Direktörü ve İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3998,14 +3915,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K85" t="str">
-        <x:v>Merhaba Yiğitcan, Aras Kargo icin İnsan ve Kültür Başkan Yardımcısı rolunuzu gordum. Logistics / Delivery tarafinda kargo dagitim ve lojistik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'kargo dagitim ve lojistik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Yiğitcan, Aras Kargo genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L85" t="str">
-        <x:v>Subject: Aras Kargo ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Aras Kargo organizasyonel İngilizce gelişim standardı
 Merhaba Yiğitcan,
-Aras Kargo ekibinin Logistics / Delivery olceginde kargo dagitim ve lojistik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: kargo dagitim ve lojistik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Aras Kargo icin mantikli pilot segmentini birlikte cikaralim.
+Aras Kargo bünyesinde Logistics / Delivery ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: kargo dagitim ve lojistik nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4043,14 +3959,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K86" t="str">
-        <x:v>Merhaba Salih, Yurtiçi Kargo icin İnsan Kaynakları ve Eğitim Genel Müdür Yardımcısı rolunuzu gordum. Logistics / Delivery tarafinda kargo ve lojistik operasyonlari nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'kargo ve lojistik operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Salih, Yurtiçi Kargo için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L86" t="str">
-        <x:v>Subject: Yurtiçi Kargo ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Yurtiçi Kargo için 2 haftalık İngilizce gelişim pilotu
 Merhaba Salih,
-Yurtiçi Kargo ekibinin Logistics / Delivery olceginde kargo ve lojistik operasyonlari odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: kargo ve lojistik operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Yurtiçi Kargo icin mantikli pilot segmentini birlikte cikaralim.
+Yurtiçi Kargo liderlik ekibinde İnsan Kaynakları ve Eğitim Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4088,14 +4003,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K87" t="str">
-        <x:v>Merhaba Selim, Hyundai Assan icin İnsan Kaynakları Yönetimi Bölüm Müdürü rolunuzu gordum. Automotive / Manufacturing tarafinda otomotiv uretim ve ihracat nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Selim, Hyundai Assan genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L87" t="str">
-        <x:v>Subject: Hyundai Assan ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Hyundai Assan organizasyonel İngilizce gelişim standardı
 Merhaba Selim,
-Hyundai Assan ekibinin Automotive / Manufacturing olceginde otomotiv uretim ve ihracat odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Hyundai Assan icin mantikli pilot segmentini birlikte cikaralim.
+Hyundai Assan bünyesinde Automotive / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4133,14 +4047,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K88" t="str">
-        <x:v>Merhaba Tolga, Hyundai Assan icin İnsan Kaynakları Planlama Bölüm Müdürü rolunuzu gordum. Automotive / Manufacturing tarafinda otomotiv uretim ve ihracat nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Tolga, Hyundai Assan için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L88" t="str">
-        <x:v>Subject: Hyundai Assan ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Hyundai Assan için 2 haftalık İngilizce gelişim pilotu
 Merhaba Tolga,
-Hyundai Assan ekibinin Automotive / Manufacturing olceginde otomotiv uretim ve ihracat odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Hyundai Assan icin mantikli pilot segmentini birlikte cikaralim.
+Hyundai Assan liderlik ekibinde İnsan Kaynakları Planlama Bölüm Müdürü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4178,14 +4091,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K89" t="str">
-        <x:v>Merhaba Yakup, Kalyon Holding icin İnsan Kaynakları Grup Müdürü rolunuzu gordum. Unknown tarafinda buyuyen ekip yapisi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Yakup, Kalyon Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L89" t="str">
-        <x:v>Subject: Kalyon Holding ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Kalyon Holding organizasyonel İngilizce gelişim standardı
 Merhaba Yakup,
-Kalyon Holding ekibinin Unknown olceginde buyuyen ekip yapisi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Kalyon Holding icin mantikli pilot segmentini birlikte cikaralim.
+Kalyon Holding bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4223,14 +4135,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K90" t="str">
-        <x:v>Merhaba Ebubekir, Medicana Sağlık Grubu icin İnsan Kaynakları Direktörü rolunuzu gordum. Healthcare / Hospitals tarafinda ozel saglik ve hastane yonetimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'ozel saglik ve hastane yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Ebubekir, Medicana Sağlık Grubu için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L90" t="str">
-        <x:v>Subject: Medicana Sağlık Grubu ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Medicana Sağlık Grubu için 2 haftalık İngilizce gelişim pilotu
 Merhaba Ebubekir,
-Medicana Sağlık Grubu ekibinin Healthcare / Hospitals olceginde ozel saglik ve hastane yonetimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: ozel saglik ve hastane yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Medicana Sağlık Grubu icin mantikli pilot segmentini birlikte cikaralim.
+Medicana Sağlık Grubu liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4268,14 +4179,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K91" t="str">
-        <x:v>Merhaba Sevil, Danone Türkiye icin İnsan Kaynakları Direktörü rolunuzu gordum. FMCG / Food tarafinda global gida sirketi ve beslenme odakli buyume nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global gida sirketi ve beslenme odakli buyume nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Sevil, Danone Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L91" t="str">
-        <x:v>Subject: Danone Türkiye ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Danone Türkiye organizasyonel İngilizce gelişim standardı
 Merhaba Sevil,
-Danone Türkiye ekibinin FMCG / Food olceginde global gida sirketi ve beslenme odakli buyume odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global gida sirketi ve beslenme odakli buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Danone Türkiye icin mantikli pilot segmentini birlikte cikaralim.
+Danone Türkiye bünyesinde FMCG / Food ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global gida sirketi ve beslenme odakli buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4313,14 +4223,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K92" t="str">
-        <x:v>Merhaba Tülin, Yurtiçi Kargo icin İnsan Kaynakları Müdürü rolunuzu gordum. Logistics / Delivery tarafinda kargo ve lojistik operasyonlari nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'kargo ve lojistik operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Tülin, Yurtiçi Kargo için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L92" t="str">
-        <x:v>Subject: Yurtiçi Kargo ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Yurtiçi Kargo için 2 haftalık İngilizce gelişim pilotu
 Merhaba Tülin,
-Yurtiçi Kargo ekibinin Logistics / Delivery olceginde kargo ve lojistik operasyonlari odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: kargo ve lojistik operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Yurtiçi Kargo icin mantikli pilot segmentini birlikte cikaralim.
+Yurtiçi Kargo liderlik ekibinde İnsan Kaynakları Müdürü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4358,14 +4267,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K93" t="str">
-        <x:v>Merhaba Nilüfer, Teknosa icin İnsan Kaynakları ve Sürdürülebilirlik Genel Müdür Yardımcısı rolunuzu gordum. Retail / Electronics tarafinda teknoloji perakende ve dijital donusum nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'teknoloji perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Nilüfer, Teknosa genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L93" t="str">
-        <x:v>Subject: Teknosa ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Teknosa organizasyonel İngilizce gelişim standardı
 Merhaba Nilüfer,
-Teknosa ekibinin Retail / Electronics olceginde teknoloji perakende ve dijital donusum odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: teknoloji perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Teknosa icin mantikli pilot segmentini birlikte cikaralim.
+Teknosa bünyesinde Retail / Electronics ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: teknoloji perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4403,14 +4311,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K94" t="str">
-        <x:v>Merhaba Seçil, MediaMarkt Türkiye icin İnsan Kaynakları Direktörü ve İcra Kurulu Üyesi rolunuzu gordum. Retail / Electronics tarafinda teknoloji perakende ve MediaSaturn is birligi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'teknoloji perakende ve MediaSaturn is birligi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Seçil, MediaMarkt Türkiye için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L94" t="str">
-        <x:v>Subject: MediaMarkt Türkiye ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: MediaMarkt Türkiye için 2 haftalık İngilizce gelişim pilotu
 Merhaba Seçil,
-MediaMarkt Türkiye ekibinin Retail / Electronics olceginde teknoloji perakende ve MediaSaturn is birligi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: teknoloji perakende ve MediaSaturn is birligi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede MediaMarkt Türkiye icin mantikli pilot segmentini birlikte cikaralim.
+MediaMarkt Türkiye liderlik ekibinde İnsan Kaynakları Direktörü ve İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4448,14 +4355,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K95" t="str">
-        <x:v>Merhaba Sebla, Koton icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Retail / Fashion tarafinda hizli moda ve uluslararasi buyume nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Sebla, Koton genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L95" t="str">
-        <x:v>Subject: Koton ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Koton organizasyonel İngilizce gelişim standardı
 Merhaba Sebla,
-Koton ekibinin Retail / Fashion olceginde hizli moda ve uluslararasi buyume odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Koton icin mantikli pilot segmentini birlikte cikaralim.
+Koton bünyesinde Retail / Fashion ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4493,14 +4399,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K96" t="str">
-        <x:v>Merhaba Hüseyin, FLO Mağazacılık icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Retail / Footwear tarafinda ayakkabi perakende ve marka portfoyu nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'ayakkabi perakende ve marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Hüseyin, FLO Mağazacılık için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L96" t="str">
-        <x:v>Subject: FLO Mağazacılık ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: FLO Mağazacılık için 2 haftalık İngilizce gelişim pilotu
 Merhaba Hüseyin,
-FLO Mağazacılık ekibinin Retail / Footwear olceginde ayakkabi perakende ve marka portfoyu odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: ayakkabi perakende ve marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede FLO Mağazacılık icin mantikli pilot segmentini birlikte cikaralim.
+FLO Mağazacılık liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4538,14 +4443,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K97" t="str">
-        <x:v>Merhaba İrem, Otokoç Otomotiv icin İnsan Kaynakları, Sürdürülebilirlik ve Kalite Direktörü rolunuzu gordum. Automotive / Rental tarafinda otomotiv dagitim ve filo yonetimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'otomotiv dagitim ve filo yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam İrem, Otokoç Otomotiv genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L97" t="str">
-        <x:v>Subject: Otokoç Otomotiv ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Otokoç Otomotiv organizasyonel İngilizce gelişim standardı
 Merhaba İrem,
-Otokoç Otomotiv ekibinin Automotive / Rental olceginde otomotiv dagitim ve filo yonetimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: otomotiv dagitim ve filo yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Otokoç Otomotiv icin mantikli pilot segmentini birlikte cikaralim.
+Otokoç Otomotiv bünyesinde Automotive / Rental ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: otomotiv dagitim ve filo yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4583,14 +4487,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K98" t="str">
-        <x:v>Merhaba Selim, Penti icin Chief Operating Officer (eski İK Direktörü) rolunuzu gordum. Retail / Fashion tarafinda ic giyim perakende ve uluslararasi buyume nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'ic giyim perakende ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Selim, Penti için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L98" t="str">
-        <x:v>Subject: Penti ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Penti için 2 haftalık İngilizce gelişim pilotu
 Merhaba Selim,
-Penti ekibinin Retail / Fashion olceginde ic giyim perakende ve uluslararasi buyume odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: ic giyim perakende ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Penti icin mantikli pilot segmentini birlikte cikaralim.
+Penti liderlik ekibinde Chief Operating Officer (eski İK Direktörü) olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4628,14 +4531,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K99" t="str">
-        <x:v>Merhaba Pınar, Şekerbank icin İnsan Kaynakları Genel Müdür Yardımcısı rolunuzu gordum. Banking / Finance tarafinda KOBi bankaciligi ve tarim bankaciligi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'KOBi bankaciligi ve tarim bankaciligi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Pınar, Şekerbank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L99" t="str">
-        <x:v>Subject: Şekerbank ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Şekerbank organizasyonel İngilizce gelişim standardı
 Merhaba Pınar,
-Şekerbank ekibinin Banking / Finance olceginde KOBi bankaciligi ve tarim bankaciligi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: KOBi bankaciligi ve tarim bankaciligi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Şekerbank icin mantikli pilot segmentini birlikte cikaralim.
+Şekerbank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: KOBi bankaciligi ve tarim bankaciligi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4673,14 +4575,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K100" t="str">
-        <x:v>Merhaba Gözde, AXA Sigorta icin İnsan Kaynakları İş Ortaklığı Müdürü rolunuzu gordum. Insurance / Finance tarafinda global sigorta ve risk yonetimi nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'global sigorta ve risk yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Merhaba Gözde, AXA Sigorta için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L100" t="str">
-        <x:v>Subject: AXA Sigorta ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: AXA Sigorta için 2 haftalık İngilizce gelişim pilotu
 Merhaba Gözde,
-AXA Sigorta ekibinin Insurance / Finance olceginde global sigorta ve risk yonetimi odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: global sigorta ve risk yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede AXA Sigorta icin mantikli pilot segmentini birlikte cikaralim.
+AXA Sigorta liderlik ekibinde İnsan Kaynakları İş Ortaklığı Müdürü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
+Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4718,14 +4619,13 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K101" t="str">
-        <x:v>Merhaba Özgür, Türk Traktör icin İnsan Kaynakları Direktörü rolunuzu gordum. Agricultural machinery / Manufacturing tarafinda tarim makineleri ve muhendislik nedeniyle Ingilizce iletisim kritik hale geliyor. Konusarak Ogren'de 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' basligiyla 2 haftalik kucuk bir pilot kurguluyoruz. Eger 'tarim makineleri ve muhendislik nedeniyle Ingilizce gelisim programini olceklendirmek' gundeminizdeyse 15 dk fikir alisverisi yapmak isterim.</x:v>
+        <x:v>Selam Özgür, Türk Traktör genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
       </x:c>
       <x:c r="L101" t="str">
-        <x:v>Subject: Türk Traktör ekipleri icin konusma odakli Ingilizce pilotu
+        <x:v>Subject: Türk Traktör organizasyonel İngilizce gelişim standardı
 Merhaba Özgür,
-Türk Traktör ekibinin Agricultural machinery / Manufacturing olceginde tarim makineleri ve muhendislik odagi oldugunu goruyorum. Bu yapidaki HR ekiplerinde sik gordugumuz konu: tarim makineleri ve muhendislik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Konusarak Ogren ile 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' uzerine dusuk eforlu bir pilot tasarlayabiliriz: seviye tespiti, hedef grup secimi, konusma pratigi ve kisa gelisim raporu.
-Uygunsa bu hafta 15 dakikalik bir gorusmede Türk Traktör icin mantikli pilot segmentini birlikte cikaralim.
+Türk Traktör bünyesinde Agricultural machinery / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: tarim makineleri ve muhendislik nedeniyle Ingilizce gelisim programini olceklendirmek.
+Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>

</xml_diff>

<commit_message>
fix: support Turkish characters and keywords in seniority and persona classification
</commit_message>
<xml_diff>
--- a/output/konusarak-ogren-hr-outbound-google-sheets.xlsx
+++ b/output/konusarak-ogren-hr-outbound-google-sheets.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HR Leads" sheetId="1" r:id="R2aa12f7f10b44b85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="2" r:id="R6e8121f6ab5d499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HR Leads" sheetId="1" r:id="Reb735e8449d14e9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="2" r:id="R8905e8d51c874a74"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -254,27 +254,27 @@
         <x:v>5000+</x:v>
       </x:c>
       <x:c r="H2" t="str">
-        <x:v>global bankacilik standartlari ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek</x:v>
+        <x:v>Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak</x:v>
       </x:c>
       <x:c r="I2" t="str">
         <x:v>86</x:v>
       </x:c>
       <x:c r="J2" t="str">
-        <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
+        <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K2" t="str">
-        <x:v>Merhaba Ebru, Garanti BBVA için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Ebru, çalışan bağlılığını artırmak için Garanti BBVA ekibine esnek konuşma pratiği faydası sunuyoruz. 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgumuzu incelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>Subject: Garanti BBVA için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Garanti BBVA çalışan deneyimi: İngilizce gelişim yan hakkı
 Merhaba Ebru,
-Garanti BBVA liderlik ekibinde Yetenek ve Kültür Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+Son dönemde çalışan bağlılığını artırmak için en çok tercih edilen yan haklardan biri yabancı dil gelişimi. Garanti BBVA ekiplerinde de bu deneyimi iyileştirmek istediğinizi biliyoruz.
+Esnek ders saatleriyle çalışanların severek kullanacağı 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelini tasarladık. Çalışan memnuniyetine etkisi üzerine konuşmak isterseniz 10 dakika zamanınızı rica edebilir miyim?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M2" t="str">
-        <x:v>86</x:v>
+        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -298,27 +298,27 @@
         <x:v>5000+</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>dijital bankacilik ve yetenek donusumu nedeniyle Ingilizce gelisim programini olceklendirmek</x:v>
+        <x:v>Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak</x:v>
       </x:c>
       <x:c r="I3" t="str">
         <x:v>83</x:v>
       </x:c>
       <x:c r="J3" t="str">
-        <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
+        <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>Selam Bülent, Akbank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Bülent, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L3" t="str">
-        <x:v>Subject: Akbank organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Akbank çalışan bağlılığı ve kişisel gelişim fırsatları
 Merhaba Bülent,
-Akbank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: dijital bankacilik ve yetenek donusumu nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M3" t="str">
-        <x:v>83</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -362,7 +362,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M4" t="str">
-        <x:v>81</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -406,7 +406,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M5" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -450,7 +450,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M6" t="str">
-        <x:v>80</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -494,7 +494,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M7" t="str">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -538,7 +538,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M8" t="str">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -582,7 +582,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M9" t="str">
-        <x:v>75</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -626,7 +626,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M10" t="str">
-        <x:v>74</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -670,7 +670,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M11" t="str">
-        <x:v>74</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -694,27 +694,27 @@
         <x:v>5000+</x:v>
       </x:c>
       <x:c r="H12" t="str">
-        <x:v>kurumsal performans ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek</x:v>
+        <x:v>Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak</x:v>
       </x:c>
       <x:c r="I12" t="str">
         <x:v>76</x:v>
       </x:c>
       <x:c r="J12" t="str">
-        <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
+        <x:v>L&amp;D programlarina olculebilir konusma pratigi katmani</x:v>
       </x:c>
       <x:c r="K12" t="str">
-        <x:v>Merhaba Şuayyip, VakıfBank için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Şuayyip, VakıfBank L&amp;D süreçlerinde katılımı artıracak konuşma odaklı İngilizce eğitimi tasarlıyoruz. Gündeminizde 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' varsa kısa bir görüşme planlayabiliriz.</x:v>
       </x:c>
       <x:c r="L12" t="str">
-        <x:v>Subject: VakıfBank için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: VakıfBank L&amp;D: Konuşma odaklı İngilizce gelişiminde ROI
 Merhaba Şuayyip,
-VakıfBank liderlik ekibinde İnsan Kaynakları, Kurumsal Gelişim ve Performans Yönetimi GMY olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+Geleneksel kurumsal İngilizce eğitimlerinde katılım ve tamamlanma oranları genellikle düşük kalıyor. L&amp;D lideri olarak hedefinizin 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' olduğunu tahmin ediyorum.
+Konusarak Ogren olarak geliştirdiğimiz birebir konuşma pratiği modeliyle katılım oranlarını %85'in üzerine çıkarıyoruz. VakıfBank ekipleri için 'L&amp;D programlarina olculebilir konusma pratigi katmani' üzerine konuşmak için önümüzdeki hafta uygun musunuz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M12" t="str">
-        <x:v>76</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -758,7 +758,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M13" t="str">
-        <x:v>76</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -802,7 +802,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M14" t="str">
-        <x:v>84</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -846,7 +846,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M15" t="str">
-        <x:v>89</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -870,27 +870,27 @@
         <x:v>1000-5000</x:v>
       </x:c>
       <x:c r="H16" t="str">
-        <x:v>katilim bankaciligi ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek</x:v>
+        <x:v>Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak</x:v>
       </x:c>
       <x:c r="I16" t="str">
         <x:v>72</x:v>
       </x:c>
       <x:c r="J16" t="str">
-        <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
+        <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K16" t="str">
-        <x:v>Merhaba Lütfü, Albaraka Türk için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Lütfü, çalışan bağlılığını artırmak için Albaraka Türk ekibine esnek konuşma pratiği faydası sunuyoruz. 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgumuzu incelemek ister misiniz?</x:v>
       </x:c>
       <x:c r="L16" t="str">
-        <x:v>Subject: Albaraka Türk için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Albaraka Türk çalışan deneyimi: İngilizce gelişim yan hakkı
 Merhaba Lütfü,
-Albaraka Türk liderlik ekibinde İnsan ve Kültür Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+Son dönemde çalışan bağlılığını artırmak için en çok tercih edilen yan haklardan biri yabancı dil gelişimi. Albaraka Türk ekiplerinde de bu deneyimi iyileştirmek istediğinizi biliyoruz.
+Esnek ders saatleriyle çalışanların severek kullanacağı 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelini tasarladık. Çalışan memnuniyetine etkisi üzerine konuşmak isterseniz 10 dakika zamanınızı rica edebilir miyim?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M16" t="str">
-        <x:v>71</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -934,7 +934,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M17" t="str">
-        <x:v>77</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -978,7 +978,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M18" t="str">
-        <x:v>88</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1066,7 +1066,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M20" t="str">
-        <x:v>82</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1110,7 +1110,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M21" t="str">
-        <x:v>82</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1198,7 +1198,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M23" t="str">
-        <x:v>93</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1242,7 +1242,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M24" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1286,7 +1286,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M25" t="str">
-        <x:v>75</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1330,7 +1330,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M26" t="str">
-        <x:v>79</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1374,7 +1374,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M27" t="str">
-        <x:v>77</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1638,7 +1638,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M33" t="str">
-        <x:v>87</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -1682,7 +1682,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M34" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -1726,7 +1726,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M35" t="str">
-        <x:v>85</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -1770,7 +1770,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M36" t="str">
-        <x:v>73</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -1814,7 +1814,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M37" t="str">
-        <x:v>69</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -1858,7 +1858,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M38" t="str">
-        <x:v>72</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -1902,7 +1902,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M39" t="str">
-        <x:v>71</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -1946,7 +1946,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M40" t="str">
-        <x:v>65</x:v>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -1990,7 +1990,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M41" t="str">
-        <x:v>72</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2034,7 +2034,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M42" t="str">
-        <x:v>74</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2078,7 +2078,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M43" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2122,7 +2122,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M44" t="str">
-        <x:v>72</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2166,7 +2166,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M45" t="str">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -2210,7 +2210,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M46" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -2254,7 +2254,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M47" t="str">
-        <x:v>79</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2298,7 +2298,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M48" t="str">
-        <x:v>88</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2342,7 +2342,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M49" t="str">
-        <x:v>75</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -2386,7 +2386,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M50" t="str">
-        <x:v>77</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -2430,7 +2430,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M51" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -2474,7 +2474,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M52" t="str">
-        <x:v>79</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -2518,7 +2518,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M53" t="str">
-        <x:v>83</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -2606,7 +2606,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M55" t="str">
-        <x:v>80</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2650,7 +2650,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M56" t="str">
-        <x:v>81</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -2694,7 +2694,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M57" t="str">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -2738,7 +2738,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M58" t="str">
-        <x:v>76</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -2782,7 +2782,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M59" t="str">
-        <x:v>85</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -2826,7 +2826,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M60" t="str">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -2850,27 +2850,27 @@
         <x:v>5000+</x:v>
       </x:c>
       <x:c r="H61" t="str">
-        <x:v>enerji dagitim ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek</x:v>
+        <x:v>Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak</x:v>
       </x:c>
       <x:c r="I61" t="str">
         <x:v>80</x:v>
       </x:c>
       <x:c r="J61" t="str">
-        <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
+        <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K61" t="str">
-        <x:v>Selam Berrin, Enerjisa genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Berrin, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L61" t="str">
-        <x:v>Subject: Enerjisa organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Enerjisa çalışan bağlılığı ve kişisel gelişim fırsatları
 Merhaba Berrin,
-Enerjisa bünyesinde Energy / Utilities ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: enerji dagitim ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M61" t="str">
-        <x:v>80</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -2914,7 +2914,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M62" t="str">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -2958,7 +2958,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M63" t="str">
-        <x:v>73</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -3002,7 +3002,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M64" t="str">
-        <x:v>89</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -3046,7 +3046,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M65" t="str">
-        <x:v>91</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -3134,7 +3134,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M67" t="str">
-        <x:v>87</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -3178,7 +3178,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M68" t="str">
-        <x:v>82</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -3222,7 +3222,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M69" t="str">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -3266,7 +3266,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M70" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -3310,7 +3310,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M71" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3354,7 +3354,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M72" t="str">
-        <x:v>84</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -3398,7 +3398,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M73" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -3442,7 +3442,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M74" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -3486,7 +3486,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M75" t="str">
-        <x:v>80</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -3530,7 +3530,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M76" t="str">
-        <x:v>79</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -3574,7 +3574,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M77" t="str">
-        <x:v>77</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -3618,7 +3618,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M78" t="str">
-        <x:v>77</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -3662,7 +3662,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M79" t="str">
-        <x:v>79</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -3706,7 +3706,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M80" t="str">
-        <x:v>72</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -3750,7 +3750,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M81" t="str">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -3794,7 +3794,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M82" t="str">
-        <x:v>80</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -3838,7 +3838,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M83" t="str">
-        <x:v>77</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -3882,7 +3882,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M84" t="str">
-        <x:v>81</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -3906,27 +3906,27 @@
         <x:v>5000+</x:v>
       </x:c>
       <x:c r="H85" t="str">
-        <x:v>kargo dagitim ve lojistik nedeniyle Ingilizce gelisim programini olceklendirmek</x:v>
+        <x:v>Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak</x:v>
       </x:c>
       <x:c r="I85" t="str">
         <x:v>70</x:v>
       </x:c>
       <x:c r="J85" t="str">
-        <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
+        <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K85" t="str">
-        <x:v>Selam Yiğitcan, Aras Kargo genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Yiğitcan, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L85" t="str">
-        <x:v>Subject: Aras Kargo organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Aras Kargo çalışan bağlılığı ve kişisel gelişim fırsatları
 Merhaba Yiğitcan,
-Aras Kargo bünyesinde Logistics / Delivery ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: kargo dagitim ve lojistik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M85" t="str">
-        <x:v>70</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -3950,27 +3950,27 @@
         <x:v>5000+</x:v>
       </x:c>
       <x:c r="H86" t="str">
-        <x:v>kargo ve lojistik operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek</x:v>
+        <x:v>Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak</x:v>
       </x:c>
       <x:c r="I86" t="str">
         <x:v>68</x:v>
       </x:c>
       <x:c r="J86" t="str">
-        <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
+        <x:v>L&amp;D programlarina olculebilir konusma pratigi katmani</x:v>
       </x:c>
       <x:c r="K86" t="str">
-        <x:v>Merhaba Salih, Yurtiçi Kargo için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Salih, Yurtiçi Kargo L&amp;D süreçlerinde katılımı artıracak konuşma odaklı İngilizce eğitimi tasarlıyoruz. Gündeminizde 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' varsa kısa bir görüşme planlayabiliriz.</x:v>
       </x:c>
       <x:c r="L86" t="str">
-        <x:v>Subject: Yurtiçi Kargo için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Yurtiçi Kargo L&amp;D: Konuşma odaklı İngilizce gelişiminde ROI
 Merhaba Salih,
-Yurtiçi Kargo liderlik ekibinde İnsan Kaynakları ve Eğitim Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+Geleneksel kurumsal İngilizce eğitimlerinde katılım ve tamamlanma oranları genellikle düşük kalıyor. L&amp;D lideri olarak hedefinizin 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' olduğunu tahmin ediyorum.
+Konusarak Ogren olarak geliştirdiğimiz birebir konuşma pratiği modeliyle katılım oranlarını %85'in üzerine çıkarıyoruz. Yurtiçi Kargo ekipleri için 'L&amp;D programlarina olculebilir konusma pratigi katmani' üzerine konuşmak için önümüzdeki hafta uygun musunuz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M86" t="str">
-        <x:v>68</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -4014,7 +4014,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M87" t="str">
-        <x:v>75</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -4058,7 +4058,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M88" t="str">
-        <x:v>75</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -4102,7 +4102,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M89" t="str">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -4146,7 +4146,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M90" t="str">
-        <x:v>72</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -4190,7 +4190,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M91" t="str">
-        <x:v>85</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -4234,7 +4234,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M92" t="str">
-        <x:v>68</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -4278,7 +4278,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M93" t="str">
-        <x:v>73</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -4322,7 +4322,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M94" t="str">
-        <x:v>77</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -4366,7 +4366,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M95" t="str">
-        <x:v>70</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -4410,7 +4410,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M96" t="str">
-        <x:v>68</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -4454,7 +4454,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M97" t="str">
-        <x:v>79</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -4498,7 +4498,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M98" t="str">
-        <x:v>69</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -4542,7 +4542,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M99" t="str">
-        <x:v>71</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -4586,7 +4586,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M100" t="str">
-        <x:v>81</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -4630,7 +4630,7 @@
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M101" t="str">
-        <x:v>75</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: resolve template repetitiveness by dynamically blending sub-templates into 700+ email variations
</commit_message>
<xml_diff>
--- a/output/konusarak-ogren-hr-outbound-google-sheets.xlsx
+++ b/output/konusarak-ogren-hr-outbound-google-sheets.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HR Leads" sheetId="1" r:id="Reb735e8449d14e9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="2" r:id="R8905e8d51c874a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HR Leads" sheetId="1" r:id="R284ddada03d24f90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="2" r:id="R5e5a663afa354dbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -263,14 +263,15 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K2" t="str">
-        <x:v>Merhaba Ebru, çalışan bağlılığını artırmak için Garanti BBVA ekibine esnek konuşma pratiği faydası sunuyoruz. 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgumuzu incelemek ister misiniz?</x:v>
+        <x:v>Selamlar Ebru, Garanti BBVA İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' varsa, kurguladığımız 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>Subject: Garanti BBVA çalışan deneyimi: İngilizce gelişim yan hakkı
-Merhaba Ebru,
-Son dönemde çalışan bağlılığını artırmak için en çok tercih edilen yan haklardan biri yabancı dil gelişimi. Garanti BBVA ekiplerinde de bu deneyimi iyileştirmek istediğinizi biliyoruz.
-Esnek ders saatleriyle çalışanların severek kullanacağı 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelini tasarladık. Çalışan memnuniyetine etkisi üzerine konuşmak isterseniz 10 dakika zamanınızı rica edebilir miyim?
-Sevgiler,
+        <x:v>Subject: Garanti BBVA çalışan gelişiminde İngilizce pratik modeli
+Değerli Ebru,
+Garanti BBVA bünyesindeki Yetenek ve Kültür Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin global bankacilik standartlari ve dijitallesme odağı varken, çalışanların dil becerilerini geliştirmek (Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M2" t="str">
@@ -307,14 +308,15 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>Selam Bülent, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
+        <x:v>Selam Bülent, Akbank bünyesindeki İnsan ve Kültür Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' konusuna yönelik, geliştirdiğimiz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L3" t="str">
-        <x:v>Subject: Akbank çalışan bağlılığı ve kişisel gelişim fırsatları
+        <x:v>Subject: Akbank ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Bülent,
-Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
-Sevgiler,
+Akbank tarafındaki İK süreçlerinizi ve Banking / Finance alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunun Akbank için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M3" t="str">
@@ -351,13 +353,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>Merhaba Ali, Türkiye İş Bankası için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Ali, Türkiye İş Bankası ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L4" t="str">
-        <x:v>Subject: Türkiye İş Bankası için 2 haftalık İngilizce gelişim pilotu
-Merhaba Ali,
-Türkiye İş Bankası liderlik ekibinde Genel Müdür Yardımcısı - İnsan Kaynakları Yönetimi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Türkiye İş Bankası ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Ali,
+Genel Müdür Yardımcısı - İnsan Kaynakları Yönetimi olarak Türkiye İş Bankası ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Banking / Finance alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: kurumsal olcekte egitim standardizasyonu nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -395,14 +398,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K5" t="str">
-        <x:v>Selam Özden, Yapı Kredi genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Özden, Yapı Kredi İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L5" t="str">
-        <x:v>Subject: Yapı Kredi organizasyonel İngilizce gelişim standardı
-Merhaba Özden,
-Yapı Kredi bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Yapı Kredi için 2 haftalık İngilizce gelişim denemesi
+Değerli Özden,
+Yapı Kredi bünyesindeki İnsan Kaynakları ve Organizasyon Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin buyuyen ekip yapisi odağı varken, çalışanların dil becerilerini geliştirmek (buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M5" t="str">
@@ -439,14 +443,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K6" t="str">
-        <x:v>Merhaba Cenk, QNB Finansbank için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Cenk, QNB Finansbank bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'dijital bankacilik ve yetenek yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L6" t="str">
-        <x:v>Subject: QNB Finansbank için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: QNB Finansbank L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Cenk,
-QNB Finansbank liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+QNB Finansbank tarafındaki İK süreçlerinizi ve Banking / Finance alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'dijital bankacilik ve yetenek yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun QNB Finansbank için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M6" t="str">
@@ -483,13 +488,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K7" t="str">
-        <x:v>Selam Tuba, DenizBank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Tuba, DenizBank ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L7" t="str">
-        <x:v>Subject: DenizBank organizasyonel İngilizce gelişim standardı
-Merhaba Tuba,
-DenizBank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: perakende bankacilik ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: DenizBank ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Tuba,
+İnsan Kaynakları Grubu Genel Müdür Yardımcısı olarak DenizBank ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Banking / Finance alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: perakende bankacilik ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -527,14 +533,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K8" t="str">
-        <x:v>Merhaba Çiğdem, TEB için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Çiğdem, TEB İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'kurumsal bankacilik ve BNP Paribas is birligi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L8" t="str">
-        <x:v>Subject: TEB için 2 haftalık İngilizce gelişim pilotu
-Merhaba Çiğdem,
-TEB liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: TEB çalışan gelişiminde İngilizce pratik modeli
+Değerli Çiğdem,
+TEB bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin kurumsal bankacilik ve BNP Paribas is birligi odağı varken, çalışanların dil becerilerini geliştirmek (kurumsal bankacilik ve BNP Paribas is birligi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M8" t="str">
@@ -571,14 +578,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K9" t="str">
-        <x:v>Selam Hüseyin, Ziraat Bankası genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Hüseyin, Ziraat Bankası bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'kamu bankaciligi ve modernizasyon nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L9" t="str">
-        <x:v>Subject: Ziraat Bankası organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Ziraat Bankası ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Hüseyin,
-Ziraat Bankası bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: kamu bankaciligi ve modernizasyon nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Ziraat Bankası tarafındaki İK süreçlerinizi ve Banking / Finance alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'kamu bankaciligi ve modernizasyon nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Ziraat Bankası için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M9" t="str">
@@ -615,13 +623,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K10" t="str">
-        <x:v>Merhaba Caner, Halkbank için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Caner, Halkbank ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L10" t="str">
-        <x:v>Subject: Halkbank için 2 haftalık İngilizce gelişim pilotu
-Merhaba Caner,
-Halkbank liderlik ekibinde İnsan Kaynakları ve İletişim Grup Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Halkbank ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Caner,
+İnsan Kaynakları ve İletişim Grup Başkanı olarak Halkbank ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Banking / Finance alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -659,14 +668,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>Selam Neşe, Halkbank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Neşe, Halkbank İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L11" t="str">
-        <x:v>Subject: Halkbank organizasyonel İngilizce gelişim standardı
-Merhaba Neşe,
-Halkbank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Halkbank için 2 haftalık İngilizce gelişim denemesi
+Değerli Neşe,
+Halkbank bünyesindeki İnsan Kaynakları Daire Başkanı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin KOBi bankaciligi ve dijitallesme odağı varken, çalışanların dil becerilerini geliştirmek (KOBi bankaciligi ve dijitallesme nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M11" t="str">
@@ -703,14 +713,15 @@
         <x:v>L&amp;D programlarina olculebilir konusma pratigi katmani</x:v>
       </x:c>
       <x:c r="K12" t="str">
-        <x:v>Merhaba Şuayyip, VakıfBank L&amp;D süreçlerinde katılımı artıracak konuşma odaklı İngilizce eğitimi tasarlıyoruz. Gündeminizde 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' varsa kısa bir görüşme planlayabiliriz.</x:v>
+        <x:v>Selam Şuayyip, VakıfBank bünyesindeki İnsan Kaynakları, Kurumsal Gelişim ve Performans Yönetimi GMY rolünüzü gördüm. Ekiplerde yaşanan 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' konusuna yönelik, geliştirdiğimiz 'L&amp;D programlarina olculebilir konusma pratigi katmani' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L12" t="str">
-        <x:v>Subject: VakıfBank L&amp;D: Konuşma odaklı İngilizce gelişiminde ROI
+        <x:v>Subject: VakıfBank L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Şuayyip,
-Geleneksel kurumsal İngilizce eğitimlerinde katılım ve tamamlanma oranları genellikle düşük kalıyor. L&amp;D lideri olarak hedefinizin 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' olduğunu tahmin ediyorum.
-Konusarak Ogren olarak geliştirdiğimiz birebir konuşma pratiği modeliyle katılım oranlarını %85'in üzerine çıkarıyoruz. VakıfBank ekipleri için 'L&amp;D programlarina olculebilir konusma pratigi katmani' üzerine konuşmak için önümüzdeki hafta uygun musunuz?
-Sevgiler,
+VakıfBank tarafındaki İK süreçlerinizi ve Banking / Finance alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'L&amp;D programlarina olculebilir konusma pratigi katmani' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'L&amp;D programlarina olculebilir konusma pratigi katmani' kurgusunun VakıfBank için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M12" t="str">
@@ -747,13 +758,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K13" t="str">
-        <x:v>Selam Ömer, VakıfBank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Ömer, VakıfBank ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L13" t="str">
-        <x:v>Subject: VakıfBank organizasyonel İngilizce gelişim standardı
-Merhaba Ömer,
-VakıfBank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: kurumsal performans ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: VakıfBank ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Ömer,
+İnsan Kaynakları Başkanı olarak VakıfBank ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Banking / Finance alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: kurumsal performans ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -791,14 +803,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K14" t="str">
-        <x:v>Merhaba Hale, ING Türkiye için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Hale, ING Türkiye İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'global standartlar ve dijital bankacilik nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L14" t="str">
-        <x:v>Subject: ING Türkiye için 2 haftalık İngilizce gelişim pilotu
-Merhaba Hale,
-ING Türkiye liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı ve İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: ING Türkiye çalışan gelişiminde İngilizce pratik modeli
+Değerli Hale,
+ING Türkiye bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı ve İcra Kurulu Üyesi pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin global standartlar ve dijital bankacilik odağı varken, çalışanların dil becerilerini geliştirmek (global standartlar ve dijital bankacilik nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M14" t="str">
@@ -835,14 +848,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K15" t="str">
-        <x:v>Selam Funda, HSBC Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Funda, HSBC Türkiye bünyesindeki İnsan Kaynakları ve Kurumsal İletişim Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'uluslararasi bankacilik ve global ekipler nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L15" t="str">
-        <x:v>Subject: HSBC Türkiye organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: HSBC Türkiye ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Funda,
-HSBC Türkiye bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: uluslararasi bankacilik ve global ekipler nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+HSBC Türkiye tarafındaki İK süreçlerinizi ve Banking / Finance alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'uluslararasi bankacilik ve global ekipler nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun HSBC Türkiye için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M15" t="str">
@@ -879,13 +893,14 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K16" t="str">
-        <x:v>Merhaba Lütfü, çalışan bağlılığını artırmak için Albaraka Türk ekibine esnek konuşma pratiği faydası sunuyoruz. 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgumuzu incelemek ister misiniz?</x:v>
+        <x:v>Merhaba Lütfü, Albaraka Türk ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L16" t="str">
-        <x:v>Subject: Albaraka Türk çalışan deneyimi: İngilizce gelişim yan hakkı
-Merhaba Lütfü,
-Son dönemde çalışan bağlılığını artırmak için en çok tercih edilen yan haklardan biri yabancı dil gelişimi. Albaraka Türk ekiplerinde de bu deneyimi iyileştirmek istediğinizi biliyoruz.
-Esnek ders saatleriyle çalışanların severek kullanacağı 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelini tasarladık. Çalışan memnuniyetine etkisi üzerine konuşmak isterseniz 10 dakika zamanınızı rica edebilir miyim?
+        <x:v>Subject: Albaraka Türk ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Lütfü,
+İnsan ve Kültür Genel Müdür Yardımcısı olarak Albaraka Türk ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Banking / Finance alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Ekiplerinize özel tasarlayacağımız 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -923,14 +938,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K17" t="str">
-        <x:v>Selam Bike, Alternatif Bank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Bike, Alternatif Bank İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'ticari bankacilik ve yenilikci urunler nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L17" t="str">
-        <x:v>Subject: Alternatif Bank organizasyonel İngilizce gelişim standardı
-Merhaba Bike,
-Alternatif Bank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: ticari bankacilik ve yenilikci urunler nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Alternatif Bank için 2 haftalık İngilizce gelişim denemesi
+Değerli Bike,
+Alternatif Bank bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin ticari bankacilik ve yenilikci urunler odağı varken, çalışanların dil becerilerini geliştirmek (ticari bankacilik ve yenilikci urunler nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M17" t="str">
@@ -967,14 +983,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K18" t="str">
-        <x:v>Merhaba Beti, Trendyol için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Beti, Trendyol bünyesindeki İnsan Kaynakları Başkanı (CHRO) rolünüzü gördüm. Ekiplerde yaşanan 'hizli olceklenen ekipler ve uluslararasi operasyon nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L18" t="str">
-        <x:v>Subject: Trendyol için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Trendyol L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Beti,
-Trendyol liderlik ekibinde İnsan Kaynakları Başkanı (CHRO) olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+Trendyol tarafındaki İK süreçlerinizi ve E-commerce / Marketplace alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'hizli olceklenen ekipler ve uluslararasi operasyon nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Trendyol için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M18" t="str">
@@ -1011,13 +1028,14 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K19" t="str">
-        <x:v>Selam Tuğçe, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
+        <x:v>Merhaba Tuğçe, Trendyol ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L19" t="str">
-        <x:v>Subject: Trendyol çalışan bağlılığı ve kişisel gelişim fırsatları
-Merhaba Tuğçe,
-Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
+        <x:v>Subject: Trendyol ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Tuğçe,
+People and Culture Leader olarak Trendyol ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle E-commerce / Marketplace alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Ekiplerinize özel tasarlayacağımız 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1055,14 +1073,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K20" t="str">
-        <x:v>Merhaba Esra, Hepsiburada için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Esra, Hepsiburada İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'e-ticaret buyumesi ve teknoloji yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L20" t="str">
-        <x:v>Subject: Hepsiburada için 2 haftalık İngilizce gelişim pilotu
-Merhaba Esra,
-Hepsiburada liderlik ekibinde İnsan Kaynakları Grup Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Hepsiburada çalışan gelişiminde İngilizce pratik modeli
+Değerli Esra,
+Hepsiburada bünyesindeki İnsan Kaynakları Grup Başkanı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin e-ticaret buyumesi ve teknoloji yatirimlari odağı varken, çalışanların dil becerilerini geliştirmek (e-ticaret buyumesi ve teknoloji yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M20" t="str">
@@ -1099,14 +1118,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K21" t="str">
-        <x:v>Selam Petek, Getir genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Petek, Getir bünyesindeki İnsandan Sorumlu Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'cok lokasyonlu operasyon ve saha ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L21" t="str">
-        <x:v>Subject: Getir organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Getir ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Petek,
-Getir bünyesinde Quick commerce / Delivery ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: cok lokasyonlu operasyon ve saha ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Getir tarafındaki İK süreçlerinizi ve Quick commerce / Delivery alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'cok lokasyonlu operasyon ve saha ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Getir için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M21" t="str">
@@ -1143,13 +1163,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K22" t="str">
-        <x:v>Merhaba Alev, Dream Games için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Alev, Dream Games ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L22" t="str">
-        <x:v>Subject: Dream Games için 2 haftalık İngilizce gelişim pilotu
-Merhaba Alev,
-Dream Games liderlik ekibinde HR Director olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Dream Games ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Alev,
+HR Director olarak Dream Games ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Gaming / Technology alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: global urun ekipleri ve hizli ise alim nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1187,14 +1208,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K23" t="str">
-        <x:v>Selam Eda, Peak Games genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Eda, Peak Games İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'global urun ve cok uluslu calisma ritmi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L23" t="str">
-        <x:v>Subject: Peak Games organizasyonel İngilizce gelişim standardı
-Merhaba Eda,
-Peak Games bünyesinde Gaming / Technology ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global urun ve cok uluslu calisma ritmi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Peak Games için 2 haftalık İngilizce gelişim denemesi
+Değerli Eda,
+Peak Games bünyesindeki İnsan Kaynakları Direktörü pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin global urun ve cok uluslu calisma ritmi odağı varken, çalışanların dil becerilerini geliştirmek (global urun ve cok uluslu calisma ritmi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M23" t="str">
@@ -1231,14 +1253,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K24" t="str">
-        <x:v>Merhaba Nebahat, Logo Yazılım için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Nebahat, Logo Yazılım bünyesindeki Grup İnsan ve Organizasyonel Dönüşüm Direktörü rolünüzü gördüm. Ekiplerde yaşanan 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L24" t="str">
-        <x:v>Subject: Logo Yazılım için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Logo Yazılım L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Nebahat,
-Logo Yazılım liderlik ekibinde Grup İnsan ve Organizasyonel Dönüşüm Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+Logo Yazılım tarafındaki İK süreçlerinizi ve Unknown alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Logo Yazılım için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M24" t="str">
@@ -1275,13 +1298,14 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K25" t="str">
-        <x:v>Selam Aşkın, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
+        <x:v>Merhaba Aşkın, Yemeksepeti ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L25" t="str">
-        <x:v>Subject: Yemeksepeti çalışan bağlılığı ve kişisel gelişim fırsatları
-Merhaba Aşkın,
-Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
+        <x:v>Subject: Yemeksepeti ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Aşkın,
+Head of People olarak Yemeksepeti ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Food delivery / Tech alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Ekiplerinize özel tasarlayacağımız 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1319,14 +1343,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K26" t="str">
-        <x:v>Merhaba Güntülü, Sahibinden.com için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Güntülü, Sahibinden.com İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'dijital pazar yeri ve teknoloji ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L26" t="str">
-        <x:v>Subject: Sahibinden.com için 2 haftalık İngilizce gelişim pilotu
-Merhaba Güntülü,
-Sahibinden.com liderlik ekibinde İnsan ve Sürdürülebilirlik Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Sahibinden.com çalışan gelişiminde İngilizce pratik modeli
+Değerli Güntülü,
+Sahibinden.com bünyesindeki İnsan ve Sürdürülebilirlik Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin dijital pazar yeri ve teknoloji ekipleri odağı varken, çalışanların dil becerilerini geliştirmek (dijital pazar yeri ve teknoloji ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M26" t="str">
@@ -1363,14 +1388,15 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K27" t="str">
-        <x:v>Selam Gözde, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
+        <x:v>Selam Gözde, BiTaksi bünyesindeki Head of People rolünüzü gördüm. Ekiplerde yaşanan 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' konusuna yönelik, geliştirdiğimiz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L27" t="str">
-        <x:v>Subject: BiTaksi çalışan bağlılığı ve kişisel gelişim fırsatları
+        <x:v>Subject: BiTaksi ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Gözde,
-Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
-Sevgiler,
+BiTaksi tarafındaki İK süreçlerinizi ve Mobility / Technology alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunun BiTaksi için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M27" t="str">
@@ -1407,13 +1433,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K28" t="str">
-        <x:v>Merhaba Tolga, Colendi için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Tolga, Colendi ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L28" t="str">
-        <x:v>Subject: Colendi için 2 haftalık İngilizce gelişim pilotu
-Merhaba Tolga,
-Colendi liderlik ekibinde HR Advisor to CEO olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Colendi ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Tolga,
+HR Advisor to CEO olarak Colendi ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Fintech alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: uluslararasi fintech urunlesmesi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1451,14 +1478,15 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K29" t="str">
-        <x:v>Selam Dilara, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
+        <x:v>Selamlar Dilara, Papara İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak' varsa, kurguladığımız 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L29" t="str">
-        <x:v>Subject: Papara çalışan bağlılığı ve kişisel gelişim fırsatları
-Merhaba Dilara,
-Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
-Sevgiler,
+        <x:v>Subject: Papara için 2 haftalık İngilizce gelişim denemesi
+Değerli Dilara,
+Papara bünyesindeki Senior People Partner pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin fintech buyumesi ve regulasyonla uyumlu ekipler odağı varken, çalışanların dil becerilerini geliştirmek (Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M29" t="str">
@@ -1495,14 +1523,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K30" t="str">
-        <x:v>Merhaba Seda, AloTech için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Seda, AloTech bünyesindeki CHRO rolünüzü gördüm. Ekiplerde yaşanan 'musteri deneyimi teknolojisi nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L30" t="str">
-        <x:v>Subject: AloTech için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: AloTech L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Seda,
-AloTech liderlik ekibinde CHRO olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+AloTech tarafındaki İK süreçlerinizi ve B2B SaaS / Technology alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'musteri deneyimi teknolojisi nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun AloTech için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M30" t="str">
@@ -1539,13 +1568,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K31" t="str">
-        <x:v>Selam Murat, Papel genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Murat, Papel ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L31" t="str">
-        <x:v>Subject: Papel organizasyonel İngilizce gelişim standardı
-Merhaba Murat,
-Papel bünyesinde Fintech ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: dijital odeme ve fintech buyumesi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: Papel ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Murat,
+CHRO olarak Papel ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Fintech alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: dijital odeme ve fintech buyumesi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1583,14 +1613,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K32" t="str">
-        <x:v>Merhaba Selin, Bilyoner için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Selin, Bilyoner İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'dijital bahis ve teknoloji ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L32" t="str">
-        <x:v>Subject: Bilyoner için 2 haftalık İngilizce gelişim pilotu
-Merhaba Selin,
-Bilyoner liderlik ekibinde CHRO olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Bilyoner çalışan gelişiminde İngilizce pratik modeli
+Değerli Selin,
+Bilyoner bünyesindeki CHRO pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin dijital bahis ve teknoloji ekipleri odağı varken, çalışanların dil becerilerini geliştirmek (dijital bahis ve teknoloji ekipleri nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M32" t="str">
@@ -1627,14 +1658,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K33" t="str">
-        <x:v>Selam Erkan, Turkcell genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Erkan, Turkcell bünyesindeki İnsan ve İş Destekten Sorumlu Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'kurumsal donusum ve teknoloji yetkinlikleri nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L33" t="str">
-        <x:v>Subject: Turkcell organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Turkcell ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Erkan,
-Turkcell bünyesinde Telecommunications ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: kurumsal donusum ve teknoloji yetkinlikleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Turkcell tarafındaki İK süreçlerinizi ve Telecommunications alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'kurumsal donusum ve teknoloji yetkinlikleri nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Turkcell için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M33" t="str">
@@ -1671,13 +1703,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K34" t="str">
-        <x:v>Merhaba Nazlı, Vodafone Türkiye için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Nazlı, Vodafone Türkiye ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L34" t="str">
-        <x:v>Subject: Vodafone Türkiye için 2 haftalık İngilizce gelişim pilotu
-Merhaba Nazlı,
-Vodafone Türkiye liderlik ekibinde İnsan Kaynaklarından Sorumlu İcra Kurulu Başkan Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Vodafone Türkiye ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Nazlı,
+İnsan Kaynaklarından Sorumlu İcra Kurulu Başkan Yardımcısı olarak Vodafone Türkiye ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Unknown alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1715,14 +1748,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K35" t="str">
-        <x:v>Selam İskender, Türk Telekom genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar İskender, Türk Telekom İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'dijital donusum ve fiber altyapi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L35" t="str">
-        <x:v>Subject: Türk Telekom organizasyonel İngilizce gelişim standardı
-Merhaba İskender,
-Türk Telekom bünyesinde Telecommunications ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: dijital donusum ve fiber altyapi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Türk Telekom için 2 haftalık İngilizce gelişim denemesi
+Değerli İskender,
+Türk Telekom bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı (CHRO) pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin dijital donusum ve fiber altyapi odağı varken, çalışanların dil becerilerini geliştirmek (dijital donusum ve fiber altyapi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M35" t="str">
@@ -1759,14 +1793,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K36" t="str">
-        <x:v>Merhaba Bahattin, LC Waikiki için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Bahattin, LC Waikiki bünyesindeki İnsan Kaynakları Genel Müdürü (CHRO) rolünüzü gördüm. Ekiplerde yaşanan 'magaza merkez ve yurt disi perakende operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L36" t="str">
-        <x:v>Subject: LC Waikiki için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: LC Waikiki L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Bahattin,
-LC Waikiki liderlik ekibinde İnsan Kaynakları Genel Müdürü (CHRO) olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+LC Waikiki tarafındaki İK süreçlerinizi ve Retail / Fashion alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'magaza merkez ve yurt disi perakende operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun LC Waikiki için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M36" t="str">
@@ -1803,13 +1838,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K37" t="str">
-        <x:v>Selam Can, Mavi genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Can, Mavi ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L37" t="str">
-        <x:v>Subject: Mavi organizasyonel İngilizce gelişim standardı
-Merhaba Can,
-Mavi bünyesinde Retail / Fashion ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: perakende ekipleri ve marka is birlikleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: Mavi ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Can,
+Chief Human Resources Officer (CHRO) olarak Mavi ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Retail / Fashion alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: perakende ekipleri ve marka is birlikleri nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1847,14 +1883,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K38" t="str">
-        <x:v>Merhaba Yeşim, DeFacto için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Yeşim, DeFacto İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L38" t="str">
-        <x:v>Subject: DeFacto için 2 haftalık İngilizce gelişim pilotu
-Merhaba Yeşim,
-DeFacto liderlik ekibinde İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: DeFacto çalışan gelişiminde İngilizce pratik modeli
+Değerli Yeşim,
+DeFacto bünyesindeki İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin hizli moda ve uluslararasi buyume odağı varken, çalışanların dil becerilerini geliştirmek (hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M38" t="str">
@@ -1891,14 +1928,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K39" t="str">
-        <x:v>Selam Yasemin, Boyner Grup genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Yasemin, Boyner Grup bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'cok kanalli perakende donusumu nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L39" t="str">
-        <x:v>Subject: Boyner Grup organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Boyner Grup ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Yasemin,
-Boyner Grup bünyesinde Retail / Department store ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: cok kanalli perakende donusumu nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Boyner Grup tarafındaki İK süreçlerinizi ve Retail / Department store alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'cok kanalli perakende donusumu nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Boyner Grup için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M39" t="str">
@@ -1935,13 +1973,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K40" t="str">
-        <x:v>Merhaba Hasan, BİM için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Hasan, BİM ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L40" t="str">
-        <x:v>Subject: BİM için 2 haftalık İngilizce gelişim pilotu
-Merhaba Hasan,
-BİM liderlik ekibinde İnsan Kaynakları Başkanı (CHRO) olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: BİM ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Hasan,
+İnsan Kaynakları Başkanı (CHRO) olarak BİM ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Retail / Discount alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: indirim perakende ve operasyonel verimlilik nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -1979,14 +2018,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K41" t="str">
-        <x:v>Selam Olcay, Migros genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Olcay, Migros İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'gida perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L41" t="str">
-        <x:v>Subject: Migros organizasyonel İngilizce gelişim standardı
-Merhaba Olcay,
-Migros bünyesinde Retail / Grocery ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: gida perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Migros için 2 haftalık İngilizce gelişim denemesi
+Değerli Olcay,
+Migros bünyesindeki İnsan Kaynakları ve Endüstri İlişkileri GMY pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin gida perakende ve dijital donusum odağı varken, çalışanların dil becerilerini geliştirmek (gida perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M41" t="str">
@@ -2023,14 +2063,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K42" t="str">
-        <x:v>Merhaba Bahar, CarrefourSA için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Bahar, CarrefourSA bünyesindeki İnsan Kaynakları ve Sürdürülebilirlik GMY rolünüzü gördüm. Ekiplerde yaşanan 'gida perakende ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L42" t="str">
-        <x:v>Subject: CarrefourSA için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: CarrefourSA L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Bahar,
-CarrefourSA liderlik ekibinde İnsan Kaynakları ve Sürdürülebilirlik GMY olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+CarrefourSA tarafındaki İK süreçlerinizi ve Retail / Grocery alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'gida perakende ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun CarrefourSA için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M42" t="str">
@@ -2067,13 +2108,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K43" t="str">
-        <x:v>Selam Tuncer, ŞOK Marketler genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Tuncer, ŞOK Marketler ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L43" t="str">
-        <x:v>Subject: ŞOK Marketler organizasyonel İngilizce gelişim standardı
-Merhaba Tuncer,
-ŞOK Marketler bünyesinde Retail / Discount ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: hizli buyuyen indirim perakende nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: ŞOK Marketler ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Tuncer,
+İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı olarak ŞOK Marketler ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Retail / Discount alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: hizli buyuyen indirim perakende nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2111,14 +2153,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K44" t="str">
-        <x:v>Merhaba Eriş, Koçtaş için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Eriş, Koçtaş İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'yapi market ve perakende operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L44" t="str">
-        <x:v>Subject: Koçtaş için 2 haftalık İngilizce gelişim pilotu
-Merhaba Eriş,
-Koçtaş liderlik ekibinde İnsan Kaynakları ve Endüstri İlişkileri GMY olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Koçtaş çalışan gelişiminde İngilizce pratik modeli
+Değerli Eriş,
+Koçtaş bünyesindeki İnsan Kaynakları ve Endüstri İlişkileri GMY pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin yapi market ve perakende operasyonlari odağı varken, çalışanların dil becerilerini geliştirmek (yapi market ve perakende operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M44" t="str">
@@ -2155,14 +2198,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K45" t="str">
-        <x:v>Selam Ali, Ford Otosan genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Ali, Ford Otosan bünyesindeki İnsan Kaynakları Direktörü rolünüzü gördüm. Ekiplerde yaşanan 'uretim, muhendislik ve global tedarik zinciri nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L45" t="str">
-        <x:v>Subject: Ford Otosan organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Ford Otosan ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Ali,
-Ford Otosan bünyesinde Automotive / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: uretim, muhendislik ve global tedarik zinciri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Ford Otosan tarafındaki İK süreçlerinizi ve Automotive / Manufacturing alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'uretim, muhendislik ve global tedarik zinciri nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Ford Otosan için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M45" t="str">
@@ -2199,13 +2243,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K46" t="str">
-        <x:v>Merhaba Orçun, TOFAŞ için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Orçun, TOFAŞ ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L46" t="str">
-        <x:v>Subject: TOFAŞ için 2 haftalık İngilizce gelişim pilotu
-Merhaba Orçun,
-TOFAŞ liderlik ekibinde İnsan Kaynakları ve Endüstriyel İlişkiler Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: TOFAŞ ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Orçun,
+İnsan Kaynakları ve Endüstriyel İlişkiler Direktörü olarak TOFAŞ ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Unknown alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2243,14 +2288,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K47" t="str">
-        <x:v>Selam Seda, Toyota Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Seda, Toyota Türkiye İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'uretim ve kalite muhendisligi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L47" t="str">
-        <x:v>Subject: Toyota Türkiye organizasyonel İngilizce gelişim standardı
-Merhaba Seda,
-Toyota Türkiye bünyesinde Automotive / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: uretim ve kalite muhendisligi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Toyota Türkiye için 2 haftalık İngilizce gelişim denemesi
+Değerli Seda,
+Toyota Türkiye bünyesindeki İnsan Kaynakları ve Tesis Yönetim Direktörü pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin uretim ve kalite muhendisligi odağı varken, çalışanların dil becerilerini geliştirmek (uretim ve kalite muhendisligi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M47" t="str">
@@ -2287,14 +2333,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K48" t="str">
-        <x:v>Merhaba Betül, Mercedes-Benz Türk için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Betül, Mercedes-Benz Türk bünyesindeki İnsan Kaynakları Direktörü rolünüzü gördüm. Ekiplerde yaşanan 'premium otomotiv ve global standartlar nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L48" t="str">
-        <x:v>Subject: Mercedes-Benz Türk için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Mercedes-Benz Türk L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Betül,
-Mercedes-Benz Türk liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+Mercedes-Benz Türk tarafındaki İK süreçlerinizi ve Automotive / Manufacturing alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'premium otomotiv ve global standartlar nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Mercedes-Benz Türk için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M48" t="str">
@@ -2331,13 +2378,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K49" t="str">
-        <x:v>Selam Gökhan, Hyundai Assan genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Gökhan, Hyundai Assan ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L49" t="str">
-        <x:v>Subject: Hyundai Assan organizasyonel İngilizce gelişim standardı
-Merhaba Gökhan,
-Hyundai Assan bünyesinde Automotive / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: Hyundai Assan ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Gökhan,
+İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı olarak Hyundai Assan ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Automotive / Manufacturing alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2375,14 +2423,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K50" t="str">
-        <x:v>Merhaba Dr., Renault MAİS için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Dr., Renault MAİS İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'otomotiv dagitim ve satis nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L50" t="str">
-        <x:v>Subject: Renault MAİS için 2 haftalık İngilizce gelişim pilotu
-Merhaba Dr.,
-Renault MAİS liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Renault MAİS çalışan gelişiminde İngilizce pratik modeli
+Değerli Dr.,
+Renault MAİS bünyesindeki İnsan Kaynakları Direktörü pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin otomotiv dagitim ve satis odağı varken, çalışanların dil becerilerini geliştirmek (otomotiv dagitim ve satis nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M50" t="str">
@@ -2419,14 +2468,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K51" t="str">
-        <x:v>Selam Fikri, Arçelik genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Fikri, Arçelik bünyesindeki Kıdemli Direktör, İnsan Kaynakları rolünüzü gördüm. Ekiplerde yaşanan 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L51" t="str">
-        <x:v>Subject: Arçelik organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Arçelik ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Fikri,
-Arçelik bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Arçelik tarafındaki İK süreçlerinizi ve Unknown alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Arçelik için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M51" t="str">
@@ -2463,13 +2513,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K52" t="str">
-        <x:v>Merhaba Zeynep, Vestel için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Zeynep, Vestel ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L52" t="str">
-        <x:v>Subject: Vestel için 2 haftalık İngilizce gelişim pilotu
-Merhaba Zeynep,
-Vestel liderlik ekibinde İnsan Kaynakları Genel Müdürü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Vestel ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Zeynep,
+İnsan Kaynakları Genel Müdürü olarak Vestel ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Electronics / Manufacturing alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: ihracat agi ve teknik ekiplerin Ingilizce ihtiyaci nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2507,14 +2558,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K53" t="str">
-        <x:v>Selam Nursel, Borusan Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Nursel, Borusan Holding İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'sanayi ve hizmet sektoru yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L53" t="str">
-        <x:v>Subject: Borusan Holding organizasyonel İngilizce gelişim standardı
-Merhaba Nursel,
-Borusan Holding bünyesinde Conglomerate / Industrial ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: sanayi ve hizmet sektoru yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Borusan Holding için 2 haftalık İngilizce gelişim denemesi
+Değerli Nursel,
+Borusan Holding bünyesindeki İnsan Kaynakları ve Kurumsal İletişim Grup Başkanı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin sanayi ve hizmet sektoru yonetimi odağı varken, çalışanların dil becerilerini geliştirmek (sanayi ve hizmet sektoru yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M53" t="str">
@@ -2551,14 +2603,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K54" t="str">
-        <x:v>Merhaba Tuğba, Borusan Otomotiv için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Tuğba, Borusan Otomotiv bünyesindeki İK ve İSG'den Sorumlu İcra Kurulu Üyesi rolünüzü gördüm. Ekiplerde yaşanan 'premium otomotiv dagitim nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L54" t="str">
-        <x:v>Subject: Borusan Otomotiv için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Borusan Otomotiv L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Tuğba,
-Borusan Otomotiv liderlik ekibinde İK ve İSG'den Sorumlu İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+Borusan Otomotiv tarafındaki İK süreçlerinizi ve Automotive / Distribution alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'premium otomotiv dagitim nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Borusan Otomotiv için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M54" t="str">
@@ -2595,13 +2648,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K55" t="str">
-        <x:v>Selam Şengül, Şişecam genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Şengül, Şişecam ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L55" t="str">
-        <x:v>Subject: Şişecam organizasyonel İngilizce gelişim standardı
-Merhaba Şengül,
-Şişecam bünyesinde Glass / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: cam sanayi ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: Şişecam ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Şengül,
+İnsan Kaynakları Genel Müdür Yardımcısı olarak Şişecam ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Glass / Manufacturing alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: cam sanayi ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2639,14 +2693,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K56" t="str">
-        <x:v>Merhaba Neslihan, Kordsa için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Neslihan, Kordsa İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'endüstriyel tekstil ve global uretim nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L56" t="str">
-        <x:v>Subject: Kordsa için 2 haftalık İngilizce gelişim pilotu
-Merhaba Neslihan,
-Kordsa liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Kordsa çalışan gelişiminde İngilizce pratik modeli
+Değerli Neslihan,
+Kordsa bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin endüstriyel tekstil ve global uretim odağı varken, çalışanların dil becerilerini geliştirmek (endüstriyel tekstil ve global uretim nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M56" t="str">
@@ -2683,14 +2738,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K57" t="str">
-        <x:v>Selam Tuğba, Brisa genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Tuğba, Brisa bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'lastik uretimi ve Bridgestone is birligi nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L57" t="str">
-        <x:v>Subject: Brisa organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Brisa ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Tuğba,
-Brisa bünyesinde Tire / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: lastik uretimi ve Bridgestone is birligi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Brisa tarafındaki İK süreçlerinizi ve Tire / Manufacturing alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'lastik uretimi ve Bridgestone is birligi nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Brisa için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M57" t="str">
@@ -2727,13 +2783,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K58" t="str">
-        <x:v>Merhaba Tuncay, Doğan Holding için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Tuncay, Doğan Holding ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L58" t="str">
-        <x:v>Subject: Doğan Holding için 2 haftalık İngilizce gelişim pilotu
-Merhaba Tuncay,
-Doğan Holding liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Doğan Holding ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Tuncay,
+İnsan Kaynakları Direktörü olarak Doğan Holding ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Conglomerate / Media alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: medya enerji ve sanayi yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2771,14 +2828,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K59" t="str">
-        <x:v>Selam Abdulkerim, Türk Hava Yolları genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Abdulkerim, Türk Hava Yolları İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'global havayolu ve genis operasyon agi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L59" t="str">
-        <x:v>Subject: Türk Hava Yolları organizasyonel İngilizce gelişim standardı
-Merhaba Abdulkerim,
-Türk Hava Yolları bünyesinde Airlines / Aviation ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global havayolu ve genis operasyon agi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Türk Hava Yolları için 2 haftalık İngilizce gelişim denemesi
+Değerli Abdulkerim,
+Türk Hava Yolları bünyesindeki İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin global havayolu ve genis operasyon agi odağı varken, çalışanların dil becerilerini geliştirmek (global havayolu ve genis operasyon agi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M59" t="str">
@@ -2815,14 +2873,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K60" t="str">
-        <x:v>Merhaba Dilara, Pegasus Hava Yolları için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Dilara, Pegasus Hava Yolları bünyesindeki İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'dusuk maliyet havayolu ve hizli buyume nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L60" t="str">
-        <x:v>Subject: Pegasus Hava Yolları için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Pegasus Hava Yolları L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Dilara,
-Pegasus Hava Yolları liderlik ekibinde İnsan Kaynaklarından Sorumlu Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+Pegasus Hava Yolları tarafındaki İK süreçlerinizi ve Airlines / Aviation alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'dusuk maliyet havayolu ve hizli buyume nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Pegasus Hava Yolları için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M60" t="str">
@@ -2859,13 +2918,14 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K61" t="str">
-        <x:v>Selam Berrin, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
+        <x:v>Merhaba Berrin, Enerjisa ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L61" t="str">
-        <x:v>Subject: Enerjisa çalışan bağlılığı ve kişisel gelişim fırsatları
-Merhaba Berrin,
-Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
+        <x:v>Subject: Enerjisa ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Berrin,
+İnsan ve Kültür Bölüm Başkanı (CHRO) olarak Enerjisa ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Energy / Utilities alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Ekiplerinize özel tasarlayacağımız 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -2903,14 +2963,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K62" t="str">
-        <x:v>Merhaba Önder, TÜPRAŞ için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Önder, TÜPRAŞ İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'rafineri ve petrokimya uretimi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L62" t="str">
-        <x:v>Subject: TÜPRAŞ için 2 haftalık İngilizce gelişim pilotu
-Merhaba Önder,
-TÜPRAŞ liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: TÜPRAŞ çalışan gelişiminde İngilizce pratik modeli
+Değerli Önder,
+TÜPRAŞ bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin rafineri ve petrokimya uretimi odağı varken, çalışanların dil becerilerini geliştirmek (rafineri ve petrokimya uretimi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M62" t="str">
@@ -2947,14 +3008,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K63" t="str">
-        <x:v>Selam Gülay, Aksa Enerji genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Gülay, Aksa Enerji bünyesindeki İnsan Kaynakları Direktörü rolünüzü gördüm. Ekiplerde yaşanan 'enerji uretim ve yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L63" t="str">
-        <x:v>Subject: Aksa Enerji organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Aksa Enerji ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Gülay,
-Aksa Enerji bünyesinde Energy / Power ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: enerji uretim ve yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Aksa Enerji tarafındaki İK süreçlerinizi ve Energy / Power alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'enerji uretim ve yatirimlari nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Aksa Enerji için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M63" t="str">
@@ -2991,13 +3053,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K64" t="str">
-        <x:v>Merhaba Burcu, Unilever Türkiye için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Burcu, Unilever Türkiye ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L64" t="str">
-        <x:v>Subject: Unilever Türkiye için 2 haftalık İngilizce gelişim pilotu
-Merhaba Burcu,
-Unilever Türkiye liderlik ekibinde İnsan Kaynakları Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Unilever Türkiye ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Burcu,
+İnsan Kaynakları Başkanı olarak Unilever Türkiye ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle FMCG / Consumer goods alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: global FMCG ve cok uluslu calisma nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3035,14 +3098,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K65" t="str">
-        <x:v>Selam Mısra, P&amp;G Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Mısra, P&amp;G Türkiye İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'global standartlar ve liderlik gelisimi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L65" t="str">
-        <x:v>Subject: P&amp;G Türkiye organizasyonel İngilizce gelişim standardı
-Merhaba Mısra,
-P&amp;G Türkiye bünyesinde FMCG / Consumer goods ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global standartlar ve liderlik gelisimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: P&amp;G Türkiye için 2 haftalık İngilizce gelişim denemesi
+Değerli Mısra,
+P&amp;G Türkiye bünyesindeki Kıdemli İnsan Kaynakları Direktörü pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin global standartlar ve liderlik gelisimi odağı varken, çalışanların dil becerilerini geliştirmek (global standartlar ve liderlik gelisimi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M65" t="str">
@@ -3079,14 +3143,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K66" t="str">
-        <x:v>Merhaba Burak, Coca-Cola İçecek için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Burak, Coca-Cola İçecek bünyesindeki İnsan Kaynaklarından Sorumlu İcra Kurulu Üyesi rolünüzü gördüm. Ekiplerde yaşanan 'global marka ve cok ulkeli operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L66" t="str">
-        <x:v>Subject: Coca-Cola İçecek için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Coca-Cola İçecek L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Burak,
-Coca-Cola İçecek liderlik ekibinde İnsan Kaynaklarından Sorumlu İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+Coca-Cola İçecek tarafındaki İK süreçlerinizi ve Beverages / FMCG alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'global marka ve cok ulkeli operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Coca-Cola İçecek için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M66" t="str">
@@ -3123,13 +3188,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K67" t="str">
-        <x:v>Selam Oktay, Nestlé Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Oktay, Nestlé Türkiye ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L67" t="str">
-        <x:v>Subject: Nestlé Türkiye organizasyonel İngilizce gelişim standardı
-Merhaba Oktay,
-Nestlé Türkiye bünyesinde FMCG / Food ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global gida sirketi ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: Nestlé Türkiye ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Oktay,
+İnsan Kaynakları Direktörü olarak Nestlé Türkiye ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle FMCG / Food alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: global gida sirketi ve surdurulebilirlik nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3167,14 +3233,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K68" t="str">
-        <x:v>Merhaba Oğuzhan, Anadolu Efes için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Oğuzhan, Anadolu Efes İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'icecek sektoru ve uluslararasi operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L68" t="str">
-        <x:v>Subject: Anadolu Efes için 2 haftalık İngilizce gelişim pilotu
-Merhaba Oğuzhan,
-Anadolu Efes liderlik ekibinde Türkiye İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Anadolu Efes çalışan gelişiminde İngilizce pratik modeli
+Değerli Oğuzhan,
+Anadolu Efes bünyesindeki Türkiye İnsan Kaynakları Direktörü pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin icecek sektoru ve uluslararasi operasyonlar odağı varken, çalışanların dil becerilerini geliştirmek (icecek sektoru ve uluslararasi operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M68" t="str">
@@ -3211,14 +3278,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K69" t="str">
-        <x:v>Selam Eylem, Ülker / Yıldız Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Eylem, Ülker / Yıldız Holding bünyesindeki İnsan Kaynakları Başkan Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'gida uretimi ve global marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L69" t="str">
-        <x:v>Subject: Ülker / Yıldız Holding organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Ülker / Yıldız Holding ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Eylem,
-Ülker / Yıldız Holding bünyesinde FMCG / Food ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: gida uretimi ve global marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Ülker / Yıldız Holding tarafındaki İK süreçlerinizi ve FMCG / Food alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'gida uretimi ve global marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Ülker / Yıldız Holding için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M69" t="str">
@@ -3255,13 +3323,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K70" t="str">
-        <x:v>Merhaba Umut, Koç Holding için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Umut, Koç Holding ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L70" t="str">
-        <x:v>Subject: Koç Holding için 2 haftalık İngilizce gelişim pilotu
-Merhaba Umut,
-Koç Holding liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Koç Holding ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Umut,
+İnsan Kaynakları Direktörü olarak Koç Holding ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Unknown alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3299,14 +3368,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K71" t="str">
-        <x:v>Selam Yeşim, Sabancı Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Yeşim, Sabancı Holding İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L71" t="str">
-        <x:v>Subject: Sabancı Holding organizasyonel İngilizce gelişim standardı
-Merhaba Yeşim,
-Sabancı Holding bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Sabancı Holding için 2 haftalık İngilizce gelişim denemesi
+Değerli Yeşim,
+Sabancı Holding bünyesindeki İnsan Kaynakları ve Sürdürülebilirlik Grup Başkanı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin buyuyen ekip yapisi odağı varken, çalışanların dil becerilerini geliştirmek (buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M71" t="str">
@@ -3343,14 +3413,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K72" t="str">
-        <x:v>Merhaba Hakan, Zorlu Holding için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Hakan, Zorlu Holding bünyesindeki İnsan Kaynakları Grubu Başkanı rolünüzü gördüm. Ekiplerde yaşanan 'enerji tekstil teknoloji ve gayrimenkul nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L72" t="str">
-        <x:v>Subject: Zorlu Holding için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Zorlu Holding L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Hakan,
-Zorlu Holding liderlik ekibinde İnsan Kaynakları Grubu Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+Zorlu Holding tarafındaki İK süreçlerinizi ve Conglomerate alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'enerji tekstil teknoloji ve gayrimenkul nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Zorlu Holding için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M72" t="str">
@@ -3387,13 +3458,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K73" t="str">
-        <x:v>Selam Evrim, Eczacıbaşı Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Evrim, Eczacıbaşı Holding ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L73" t="str">
-        <x:v>Subject: Eczacıbaşı Holding organizasyonel İngilizce gelişim standardı
-Merhaba Evrim,
-Eczacıbaşı Holding bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: Eczacıbaşı Holding ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Evrim,
+İnsan Kaynakları Grup Başkanı olarak Eczacıbaşı Holding ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Unknown alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3431,14 +3503,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K74" t="str">
-        <x:v>Merhaba Özge, Kalyon Holding için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Özge, Kalyon Holding İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L74" t="str">
-        <x:v>Subject: Kalyon Holding için 2 haftalık İngilizce gelişim pilotu
-Merhaba Özge,
-Kalyon Holding liderlik ekibinde İnsan Kaynakları Grup Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Kalyon Holding çalışan gelişiminde İngilizce pratik modeli
+Değerli Özge,
+Kalyon Holding bünyesindeki İnsan Kaynakları Grup Başkanı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin buyuyen ekip yapisi odağı varken, çalışanların dil becerilerini geliştirmek (buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M74" t="str">
@@ -3475,14 +3548,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K75" t="str">
-        <x:v>Selam Melis, TAV Havalimanları genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Melis, TAV Havalimanları bünyesindeki İnsan Kaynakları Grup Başkanı (CHRO) rolünüzü gördüm. Ekiplerde yaşanan 'havalimani isletme ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L75" t="str">
-        <x:v>Subject: TAV Havalimanları organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: TAV Havalimanları ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Melis,
-TAV Havalimanları bünyesinde Aviation / Infrastructure ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: havalimani isletme ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+TAV Havalimanları tarafındaki İK süreçlerinizi ve Aviation / Infrastructure alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'havalimani isletme ve global operasyonlar nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun TAV Havalimanları için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M75" t="str">
@@ -3519,13 +3593,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K76" t="str">
-        <x:v>Merhaba Yalçın, Doğuş Otomotiv için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Yalçın, Doğuş Otomotiv ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L76" t="str">
-        <x:v>Subject: Doğuş Otomotiv için 2 haftalık İngilizce gelişim pilotu
-Merhaba Yalçın,
-Doğuş Otomotiv liderlik ekibinde İnsan Kaynakları ve Süreç Yönetimi Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Doğuş Otomotiv ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Yalçın,
+İnsan Kaynakları ve Süreç Yönetimi Direktörü olarak Doğuş Otomotiv ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Automotive / Distribution alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: otomotiv dagitim ve perakende nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3563,14 +3638,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K77" t="str">
-        <x:v>Selam Dr., Abdi İbrahim genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Dr., Abdi İbrahim İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L77" t="str">
-        <x:v>Subject: Abdi İbrahim organizasyonel İngilizce gelişim standardı
-Merhaba Dr.,
-Abdi İbrahim bünyesinde Pharma / Healthcare ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Abdi İbrahim için 2 haftalık İngilizce gelişim denemesi
+Değerli Dr.,
+Abdi İbrahim bünyesindeki İK, Kurumsal İletişim ve Sürdürülebilirlik Grup Başkanı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin ilac sanayi ve uluslararasi buyume odağı varken, çalışanların dil becerilerini geliştirmek (ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M77" t="str">
@@ -3607,14 +3683,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K78" t="str">
-        <x:v>Merhaba Ayşe, Abdi İbrahim için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Ayşe, Abdi İbrahim bünyesindeki Uluslararası Pazarlar İnsan Kaynakları Direktörü rolünüzü gördüm. Ekiplerde yaşanan 'ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L78" t="str">
-        <x:v>Subject: Abdi İbrahim için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Abdi İbrahim L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Ayşe,
-Abdi İbrahim liderlik ekibinde Uluslararası Pazarlar İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+Abdi İbrahim tarafındaki İK süreçlerinizi ve Pharma / Healthcare alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'ilac sanayi ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Abdi İbrahim için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M78" t="str">
@@ -3651,13 +3728,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K79" t="str">
-        <x:v>Selam Kader, Eczacıbaşı Sağlık genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Kader, Eczacıbaşı Sağlık ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L79" t="str">
-        <x:v>Subject: Eczacıbaşı Sağlık organizasyonel İngilizce gelişim standardı
-Merhaba Kader,
-Eczacıbaşı Sağlık bünyesinde Healthcare / Pharma ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: saglik urunleri ve ilac nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: Eczacıbaşı Sağlık ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Kader,
+İnsan Kaynakları Direktörü olarak Eczacıbaşı Sağlık ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Healthcare / Pharma alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: saglik urunleri ve ilac nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3695,14 +3773,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K80" t="str">
-        <x:v>Merhaba Demet, Medicana Sağlık Grubu için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Demet, Medicana Sağlık Grubu İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'ozel saglik ve hastane yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L80" t="str">
-        <x:v>Subject: Medicana Sağlık Grubu için 2 haftalık İngilizce gelişim pilotu
-Merhaba Demet,
-Medicana Sağlık Grubu liderlik ekibinde İnsan Kaynakları Grup Başkanı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Medicana Sağlık Grubu çalışan gelişiminde İngilizce pratik modeli
+Değerli Demet,
+Medicana Sağlık Grubu bünyesindeki İnsan Kaynakları Grup Başkanı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin ozel saglik ve hastane yonetimi odağı varken, çalışanların dil becerilerini geliştirmek (ozel saglik ve hastane yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M80" t="str">
@@ -3739,14 +3818,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K81" t="str">
-        <x:v>Selam Gökben, Acıbadem Sağlık Grubu genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Gökben, Acıbadem Sağlık Grubu bünyesindeki İnsan Kaynakları Direktör Vekili rolünüzü gördüm. Ekiplerde yaşanan 'premium saglik hizmetleri nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L81" t="str">
-        <x:v>Subject: Acıbadem Sağlık Grubu organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Acıbadem Sağlık Grubu ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Gökben,
-Acıbadem Sağlık Grubu bünyesinde Healthcare / Hospitals ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: premium saglik hizmetleri nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Acıbadem Sağlık Grubu tarafındaki İK süreçlerinizi ve Healthcare / Hospitals alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'premium saglik hizmetleri nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Acıbadem Sağlık Grubu için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M81" t="str">
@@ -3783,13 +3863,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K82" t="str">
-        <x:v>Merhaba Muhammed, ASELSAN için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Muhammed, ASELSAN ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L82" t="str">
-        <x:v>Subject: ASELSAN için 2 haftalık İngilizce gelişim pilotu
-Merhaba Muhammed,
-ASELSAN liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: ASELSAN ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Muhammed,
+İnsan Kaynakları Direktörü olarak ASELSAN ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Defense / Technology alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: savunma teknolojisi ve muhendislik nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3827,14 +3908,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K83" t="str">
-        <x:v>Selam Oğuzhan, HAVELSAN genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Oğuzhan, HAVELSAN İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'savunma yazilimi ve siber guvenlik nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L83" t="str">
-        <x:v>Subject: HAVELSAN organizasyonel İngilizce gelişim standardı
-Merhaba Oğuzhan,
-HAVELSAN bünyesinde Defense / Technology ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: savunma yazilimi ve siber guvenlik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: HAVELSAN için 2 haftalık İngilizce gelişim denemesi
+Değerli Oğuzhan,
+HAVELSAN bünyesindeki İnsan Kaynakları Direktörü pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin savunma yazilimi ve siber guvenlik odağı varken, çalışanların dil becerilerini geliştirmek (savunma yazilimi ve siber guvenlik nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M83" t="str">
@@ -3871,14 +3953,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K84" t="str">
-        <x:v>Merhaba Zeynep, AXA Sigorta için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Zeynep, AXA Sigorta bünyesindeki İnsan Kaynakları Direktörü ve İcra Kurulu Üyesi rolünüzü gördüm. Ekiplerde yaşanan 'global sigorta ve risk yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L84" t="str">
-        <x:v>Subject: AXA Sigorta için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: AXA Sigorta L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Zeynep,
-AXA Sigorta liderlik ekibinde İnsan Kaynakları Direktörü ve İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+AXA Sigorta tarafındaki İK süreçlerinizi ve Insurance / Finance alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'global sigorta ve risk yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun AXA Sigorta için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M84" t="str">
@@ -3915,13 +3998,14 @@
         <x:v>Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi</x:v>
       </x:c>
       <x:c r="K85" t="str">
-        <x:v>Selam Yiğitcan, çalışan memnuniyetini doğrudan artıran yan haklar kapsamında tasarladığımız konuşma koçu programını 2 haftalık ücretsiz pilotla test edebiliriz. Detaylar için uygun musunuz?</x:v>
+        <x:v>Merhaba Yiğitcan, Aras Kargo ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L85" t="str">
-        <x:v>Subject: Aras Kargo çalışan bağlılığı ve kişisel gelişim fırsatları
-Merhaba Yiğitcan,
-Şirket içi yetenekleri elde tutmak ve kariyer yollarını desteklemek, güçlü bir çalışan deneyiminden geçiyor. Bu noktada en çok karşılaşılan zorluk: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
-Konusarak Ogren ile sunduğumuz 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' kurgusunu ve örnek başarı hikayelerini paylaşmak isterim. Bu hafta kısa bir telefon görüşmesi yapabilir miyiz?
+        <x:v>Subject: Aras Kargo ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Yiğitcan,
+İnsan ve Kültür Başkan Yardımcısı olarak Aras Kargo ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Logistics / Delivery alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: Calisan bagliligini artiran, kisiye ozel gelisim benefit'i sunmak.
+Ekiplerinize özel tasarlayacağımız 'Calisan deneyimi benefit'i olarak esnek Ingilizce gelisimi' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -3959,14 +4043,15 @@
         <x:v>L&amp;D programlarina olculebilir konusma pratigi katmani</x:v>
       </x:c>
       <x:c r="K86" t="str">
-        <x:v>Merhaba Salih, Yurtiçi Kargo L&amp;D süreçlerinde katılımı artıracak konuşma odaklı İngilizce eğitimi tasarlıyoruz. Gündeminizde 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' varsa kısa bir görüşme planlayabiliriz.</x:v>
+        <x:v>Selamlar Salih, Yurtiçi Kargo İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' varsa, kurguladığımız 'L&amp;D programlarina olculebilir konusma pratigi katmani' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L86" t="str">
-        <x:v>Subject: Yurtiçi Kargo L&amp;D: Konuşma odaklı İngilizce gelişiminde ROI
-Merhaba Salih,
-Geleneksel kurumsal İngilizce eğitimlerinde katılım ve tamamlanma oranları genellikle düşük kalıyor. L&amp;D lideri olarak hedefinizin 'Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak' olduğunu tahmin ediyorum.
-Konusarak Ogren olarak geliştirdiğimiz birebir konuşma pratiği modeliyle katılım oranlarını %85'in üzerine çıkarıyoruz. Yurtiçi Kargo ekipleri için 'L&amp;D programlarina olculebilir konusma pratigi katmani' üzerine konuşmak için önümüzdeki hafta uygun musunuz?
-Sevgiler,
+        <x:v>Subject: Yurtiçi Kargo çalışan gelişiminde İngilizce pratik modeli
+Değerli Salih,
+Yurtiçi Kargo bünyesindeki İnsan Kaynakları ve Eğitim Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin kargo ve lojistik operasyonlari odağı varken, çalışanların dil becerilerini geliştirmek (Calisanlara olculebilir, olceklenebilir ve yogun programa uyumlu Ingilizce gelisim yolu kurmak) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'L&amp;D programlarina olculebilir konusma pratigi katmani' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M86" t="str">
@@ -4003,14 +4088,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K87" t="str">
-        <x:v>Selam Selim, Hyundai Assan genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Selim, Hyundai Assan bünyesindeki İnsan Kaynakları Yönetimi Bölüm Müdürü rolünüzü gördüm. Ekiplerde yaşanan 'otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L87" t="str">
-        <x:v>Subject: Hyundai Assan organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Hyundai Assan ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Selim,
-Hyundai Assan bünyesinde Automotive / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Hyundai Assan tarafındaki İK süreçlerinizi ve Automotive / Manufacturing alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Hyundai Assan için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M87" t="str">
@@ -4047,13 +4133,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K88" t="str">
-        <x:v>Merhaba Tolga, Hyundai Assan için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Tolga, Hyundai Assan ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L88" t="str">
-        <x:v>Subject: Hyundai Assan için 2 haftalık İngilizce gelişim pilotu
-Merhaba Tolga,
-Hyundai Assan liderlik ekibinde İnsan Kaynakları Planlama Bölüm Müdürü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: Hyundai Assan ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Tolga,
+İnsan Kaynakları Planlama Bölüm Müdürü olarak Hyundai Assan ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Automotive / Manufacturing alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: otomotiv uretim ve ihracat nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4091,14 +4178,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K89" t="str">
-        <x:v>Selam Yakup, Kalyon Holding genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Yakup, Kalyon Holding İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L89" t="str">
-        <x:v>Subject: Kalyon Holding organizasyonel İngilizce gelişim standardı
-Merhaba Yakup,
-Kalyon Holding bünyesinde Unknown ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Kalyon Holding için 2 haftalık İngilizce gelişim denemesi
+Değerli Yakup,
+Kalyon Holding bünyesindeki İnsan Kaynakları Grup Müdürü pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin buyuyen ekip yapisi odağı varken, çalışanların dil becerilerini geliştirmek (buyuyen ekip yapisi nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M89" t="str">
@@ -4135,14 +4223,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K90" t="str">
-        <x:v>Merhaba Ebubekir, Medicana Sağlık Grubu için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Ebubekir, Medicana Sağlık Grubu bünyesindeki İnsan Kaynakları Direktörü rolünüzü gördüm. Ekiplerde yaşanan 'ozel saglik ve hastane yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L90" t="str">
-        <x:v>Subject: Medicana Sağlık Grubu için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: Medicana Sağlık Grubu L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Ebubekir,
-Medicana Sağlık Grubu liderlik ekibinde İnsan Kaynakları Direktörü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+Medicana Sağlık Grubu tarafındaki İK süreçlerinizi ve Healthcare / Hospitals alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'ozel saglik ve hastane yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Medicana Sağlık Grubu için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M90" t="str">
@@ -4179,13 +4268,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K91" t="str">
-        <x:v>Selam Sevil, Danone Türkiye genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba Sevil, Danone Türkiye ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L91" t="str">
-        <x:v>Subject: Danone Türkiye organizasyonel İngilizce gelişim standardı
-Merhaba Sevil,
-Danone Türkiye bünyesinde FMCG / Food ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: global gida sirketi ve beslenme odakli buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: Danone Türkiye ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar Sevil,
+İnsan Kaynakları Direktörü olarak Danone Türkiye ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle FMCG / Food alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: global gida sirketi ve beslenme odakli buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4223,14 +4313,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K92" t="str">
-        <x:v>Merhaba Tülin, Yurtiçi Kargo için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Tülin, Yurtiçi Kargo İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'kargo ve lojistik operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L92" t="str">
-        <x:v>Subject: Yurtiçi Kargo için 2 haftalık İngilizce gelişim pilotu
-Merhaba Tülin,
-Yurtiçi Kargo liderlik ekibinde İnsan Kaynakları Müdürü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Yurtiçi Kargo çalışan gelişiminde İngilizce pratik modeli
+Değerli Tülin,
+Yurtiçi Kargo bünyesindeki İnsan Kaynakları Müdürü pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin kargo ve lojistik operasyonlari odağı varken, çalışanların dil becerilerini geliştirmek (kargo ve lojistik operasyonlari nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M92" t="str">
@@ -4267,14 +4358,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K93" t="str">
-        <x:v>Selam Nilüfer, Teknosa genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Nilüfer, Teknosa bünyesindeki İnsan Kaynakları ve Sürdürülebilirlik Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'teknoloji perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L93" t="str">
-        <x:v>Subject: Teknosa organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Teknosa ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Nilüfer,
-Teknosa bünyesinde Retail / Electronics ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: teknoloji perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Teknosa tarafındaki İK süreçlerinizi ve Retail / Electronics alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'teknoloji perakende ve dijital donusum nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Teknosa için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M93" t="str">
@@ -4311,13 +4403,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K94" t="str">
-        <x:v>Merhaba Seçil, MediaMarkt Türkiye için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Seçil, MediaMarkt Türkiye ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L94" t="str">
-        <x:v>Subject: MediaMarkt Türkiye için 2 haftalık İngilizce gelişim pilotu
-Merhaba Seçil,
-MediaMarkt Türkiye liderlik ekibinde İnsan Kaynakları Direktörü ve İcra Kurulu Üyesi olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: MediaMarkt Türkiye ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Seçil,
+İnsan Kaynakları Direktörü ve İcra Kurulu Üyesi olarak MediaMarkt Türkiye ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Retail / Electronics alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: teknoloji perakende ve MediaSaturn is birligi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4355,14 +4448,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K95" t="str">
-        <x:v>Selam Sebla, Koton genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Sebla, Koton İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L95" t="str">
-        <x:v>Subject: Koton organizasyonel İngilizce gelişim standardı
-Merhaba Sebla,
-Koton bünyesinde Retail / Fashion ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Koton için 2 haftalık İngilizce gelişim denemesi
+Değerli Sebla,
+Koton bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin hizli moda ve uluslararasi buyume odağı varken, çalışanların dil becerilerini geliştirmek (hizli moda ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M95" t="str">
@@ -4399,14 +4493,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K96" t="str">
-        <x:v>Merhaba Hüseyin, FLO Mağazacılık için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selam Hüseyin, FLO Mağazacılık bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'ayakkabi perakende ve marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L96" t="str">
-        <x:v>Subject: FLO Mağazacılık için 2 haftalık İngilizce gelişim pilotu
+        <x:v>Subject: FLO Mağazacılık L&amp;D / İK süreçlerinde İngilizce standardizasyonu
 Merhaba Hüseyin,
-FLO Mağazacılık liderlik ekibinde İnsan Kaynakları Genel Müdür Yardımcısı olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+FLO Mağazacılık tarafındaki İK süreçlerinizi ve Retail / Footwear alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'ayakkabi perakende ve marka portfoyu nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun FLO Mağazacılık için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M96" t="str">
@@ -4443,13 +4538,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K97" t="str">
-        <x:v>Selam İrem, Otokoç Otomotiv genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Merhaba İrem, Otokoç Otomotiv ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L97" t="str">
-        <x:v>Subject: Otokoç Otomotiv organizasyonel İngilizce gelişim standardı
-Merhaba İrem,
-Otokoç Otomotiv bünyesinde Automotive / Rental ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: otomotiv dagitim ve filo yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
+        <x:v>Subject: Otokoç Otomotiv ekipleri için konuşma odaklı İngilizce pilotu
+Selamlar İrem,
+İnsan Kaynakları, Sürdürülebilirlik ve Kalite Direktörü olarak Otokoç Otomotiv ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Automotive / Rental alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: otomotiv dagitim ve filo yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4487,14 +4583,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K98" t="str">
-        <x:v>Merhaba Selim, Penti için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Selamlar Selim, Penti İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'ic giyim perakende ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L98" t="str">
-        <x:v>Subject: Penti için 2 haftalık İngilizce gelişim pilotu
-Merhaba Selim,
-Penti liderlik ekibinde Chief Operating Officer (eski İK Direktörü) olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
-Sevgiler,
+        <x:v>Subject: Penti çalışan gelişiminde İngilizce pratik modeli
+Değerli Selim,
+Penti bünyesindeki Chief Operating Officer (eski İK Direktörü) pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin ic giyim perakende ve uluslararasi buyume odağı varken, çalışanların dil becerilerini geliştirmek (ic giyim perakende ve uluslararasi buyume nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M98" t="str">
@@ -4531,14 +4628,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K99" t="str">
-        <x:v>Selam Pınar, Şekerbank genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selam Pınar, Şekerbank bünyesindeki İnsan Kaynakları Genel Müdür Yardımcısı rolünüzü gördüm. Ekiplerde yaşanan 'KOBi bankaciligi ve tarim bankaciligi nedeniyle Ingilizce gelisim programini olceklendirmek' konusuna yönelik, geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' projesini paylaşmak isterim. Bağlantıda kalmak isterim.</x:v>
       </x:c>
       <x:c r="L99" t="str">
-        <x:v>Subject: Şekerbank organizasyonel İngilizce gelişim standardı
+        <x:v>Subject: Şekerbank ve Konuşarak Öğren: Kurumsal İngilizce İş Birliği
 Merhaba Pınar,
-Şekerbank bünyesinde Banking / Finance ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: KOBi bankaciligi ve tarim bankaciligi nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+Şekerbank tarafındaki İK süreçlerinizi ve Banking / Finance alanındaki sektörel başarılarınızı uzun süredir izliyorum.
+Sizin gibi büyüyen organizasyonlarda İK departmanlarının en çok odaklandığı konulardan biri olan 'KOBi bankaciligi ve tarim bankaciligi nedeniyle Ingilizce gelisim programini olceklendirmek' üzerine yenilikçi bir çözüm geliştirdik.
+Konusarak Ogren ile sunduğumuz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunu ve örnek başarı hikayelerini sizinle paylaşmak isterim. Uygunsa bu hafta 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' kurgusunun Şekerbank için nasıl bir fayda sağlayacağını konuşmak üzere kısa bir kahve sohbeti ayarlayabiliriz.
+Saygılarımla,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M99" t="str">
@@ -4575,13 +4673,14 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K100" t="str">
-        <x:v>Merhaba Gözde, AXA Sigorta için organizasyonel İngilizce gelişimini standardize edecek 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' üzerine 2 haftalık risk taşımayan ücretsiz bir pilot hazırladık. İncelemek ister misiniz?</x:v>
+        <x:v>Merhaba Gözde, AXA Sigorta ekibindeki çalışmalarınızı takip ediyorum. Dil engellerini aşarak iş verimliliğini artıran 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelimiz üzerine 10 dk konuşmak isterim. Kısa bir görüşme için uygun musunuz?</x:v>
       </x:c>
       <x:c r="L100" t="str">
-        <x:v>Subject: AXA Sigorta için 2 haftalık İngilizce gelişim pilotu
-Merhaba Gözde,
-AXA Sigorta liderlik ekibinde İnsan Kaynakları İş Ortaklığı Müdürü olarak, organizasyon genelinde İngilizce seviyesini standardize etmek ve bunu ölçülebilir kılmak istediğinizi tahmin ediyorum.
-Bu kapsamda 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' odaklı, risk barındırmayan 2 haftalık kurumsal bir pilot program kurguluyoruz. İlginizi çekerse detayları konuşmak üzere kısa bir kahve sohbeti planlayabiliriz.
+        <x:v>Subject: AXA Sigorta ekiplerinde dil bariyerini aşma kurgusu
+Selamlar Gözde,
+İnsan Kaynakları İş Ortaklığı Müdürü olarak AXA Sigorta ekibinde yürüttüğünüz çalışan gelişimi çalışmalarını inceleme fırsatım oldu.
+Özellikle Insurance / Finance alanında faaliyet gösteren firmalarda karşılaştığımız en yaygın konu: global sigorta ve risk yonetimi nedeniyle Ingilizce gelisim programini olceklendirmek.
+Ekiplerinize özel tasarlayacağımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modelini 2 haftalık ücretsiz bir deneme süreciyle test etmeye ne dersiniz? Sürecin nasıl çalıştığını gösteren kısa bir demo paylaşmamı veya 15 dakikalık bir fikir alışverişi planlamamızı ister misiniz?
 Sevgiler,
 Growth Automation Ekibi</x:v>
       </x:c>
@@ -4619,14 +4718,15 @@
         <x:v>Kurumsal Ingilizce gelisimini hizli pilotla test etme</x:v>
       </x:c>
       <x:c r="K101" t="str">
-        <x:v>Selam Özgür, Türk Traktör genelinde dil engellerini aşarak iş verimliliğini artıran konuşma pratiği modelimizi ve başarı hikayelerimizi aktarmak için 10 dk ayırabilir misiniz?</x:v>
+        <x:v>Selamlar Özgür, Türk Traktör İK ekibindeki profilinizi inceleme fırsatım oldu. Gündeminizde 'tarim makineleri ve muhendislik nedeniyle Ingilizce gelisim programini olceklendirmek' varsa, kurguladığımız 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' deneme programını aktarmak isterim. Detaylar için bu hafta zamanınız var mı?</x:v>
       </x:c>
       <x:c r="L101" t="str">
-        <x:v>Subject: Türk Traktör organizasyonel İngilizce gelişim standardı
-Merhaba Özgür,
-Türk Traktör bünyesinde Agricultural machinery / Manufacturing ölçeğinde büyürken, en sık karşılaşılan operasyonel engellerden biri dil bariyerleri olabiliyor. Özellikle: tarim makineleri ve muhendislik nedeniyle Ingilizce gelisim programini olceklendirmek.
-Geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' modeliyle şirket genelinde konuşma odaklı gelişimi nasıl hızlandırdığımızı aktarmak isterim. Önümüzdeki günlerde 10 dakika ayırmanız mümkün mü?
-Sevgiler,
+        <x:v>Subject: Türk Traktör için 2 haftalık İngilizce gelişim denemesi
+Değerli Özgür,
+Türk Traktör bünyesindeki İnsan Kaynakları Direktörü pozisyonunuzu ve ekibinizin büyüme adımlarını yakından takip ediyorum.
+Şirketinizin tarim makineleri ve muhendislik odağı varken, çalışanların dil becerilerini geliştirmek (tarim makineleri ve muhendislik nedeniyle Ingilizce gelisim programini olceklendirmek) kritik bir gündem maddesi olmalı.
+Bu yapıda geliştirdiğimiz 'Kurumsal Ingilizce gelisimini hizli pilotla test etme' yaklaşımıyla, çalışanların seviyelerine göre 1-on-1 konuşma koçları atıyoruz. Önümüzdeki günlerde bu konuyu değerlendirmek adına 10 dakikalık kısa bir telefon görüşmesi yapabilir miyiz?
+İyi çalışmalar dilerim,
 Growth Automation Ekibi</x:v>
       </x:c>
       <x:c r="M101" t="str">

</xml_diff>